<commit_message>
fix ajuste de inventario
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\mbs_backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{170CABC6-1CFF-4DF9-A19C-493E2D970009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E42931-0331-4854-81DA-5DF02DE00A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{20512AA4-7BE2-441B-A4C6-368DAF0E60CB}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="474">
   <si>
     <t>CH-DEP-0001</t>
   </si>
@@ -1521,6 +1521,9 @@
   <si>
     <t>VE-FOR-0051</t>
   </si>
+  <si>
+    <t>BR-DEP-0023</t>
+  </si>
 </sst>
 </file>
 
@@ -1577,7 +1580,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1593,12 +1596,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1632,7 +1629,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5638,6 +5635,15 @@
       </c>
     </row>
     <row r="172" spans="8:21" x14ac:dyDescent="0.25">
+      <c r="H172" t="s">
+        <v>473</v>
+      </c>
+      <c r="I172" t="s">
+        <v>18</v>
+      </c>
+      <c r="J172" t="s">
+        <v>13</v>
+      </c>
       <c r="M172" t="s">
         <v>345</v>
       </c>
@@ -5734,12 +5740,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="R148:U148"/>
-    <mergeCell ref="R164:U164"/>
-    <mergeCell ref="C148:F148"/>
-    <mergeCell ref="H132:K132"/>
-    <mergeCell ref="C132:F132"/>
-    <mergeCell ref="H148:K148"/>
     <mergeCell ref="R61:U61"/>
     <mergeCell ref="R4:U4"/>
     <mergeCell ref="M132:P132"/>
@@ -5750,6 +5750,12 @@
     <mergeCell ref="H61:K61"/>
     <mergeCell ref="M61:P61"/>
     <mergeCell ref="R132:U132"/>
+    <mergeCell ref="R148:U148"/>
+    <mergeCell ref="R164:U164"/>
+    <mergeCell ref="C148:F148"/>
+    <mergeCell ref="H132:K132"/>
+    <mergeCell ref="C132:F132"/>
+    <mergeCell ref="H148:K148"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: update inventario/db 2026-06-22 21:53:14
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\mbs_backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B271E545-CCB2-4C40-8CCA-D1D0268CC211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7A9A6A1-6F48-4AC5-A8B1-9F01594B08E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{20512AA4-7BE2-441B-A4C6-368DAF0E60CB}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="498">
   <si>
     <t>CH-DEP-0001</t>
   </si>
@@ -1568,6 +1568,33 @@
   </si>
   <si>
     <t>BL-CAS-0067</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>VE-CAS-0053</t>
+  </si>
+  <si>
+    <t>ST-CAS-0022</t>
+  </si>
+  <si>
+    <t>ESTAMPADO/TIGRE</t>
+  </si>
+  <si>
+    <t>FL-CAS-0017</t>
+  </si>
+  <si>
+    <t>BL-CAS-0068</t>
+  </si>
+  <si>
+    <t>ST-CAS-0023</t>
+  </si>
+  <si>
+    <t>VE-CAS-0054</t>
+  </si>
+  <si>
+    <t>BEIGE/LADRILLO</t>
   </si>
 </sst>
 </file>
@@ -1663,7 +1690,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1674,13 +1701,14 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1796,8 +1824,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{F5A9EFC3-A60C-4814-94C2-68A3EE6F970A}" name="Tabla4111516" displayName="Tabla4111516" ref="H151:K178" totalsRowShown="0">
-  <autoFilter ref="H151:K178" xr:uid="{F5A9EFC3-A60C-4814-94C2-68A3EE6F970A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{F5A9EFC3-A60C-4814-94C2-68A3EE6F970A}" name="Tabla4111516" displayName="Tabla4111516" ref="H155:K182" totalsRowShown="0">
+  <autoFilter ref="H155:K182" xr:uid="{F5A9EFC3-A60C-4814-94C2-68A3EE6F970A}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{21DD644A-E8AB-4338-A493-443B2953FFC7}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{DD3C90D9-E5C0-4983-BE77-6F1EE14652C7}" name="TALLA"/>
@@ -1809,8 +1837,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{826E6D02-7982-4253-94C2-5BA245328A25}" name="Tabla41115162" displayName="Tabla41115162" ref="M135:P193" totalsRowShown="0">
-  <autoFilter ref="M135:P193" xr:uid="{826E6D02-7982-4253-94C2-5BA245328A25}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{826E6D02-7982-4253-94C2-5BA245328A25}" name="Tabla41115162" displayName="Tabla41115162" ref="M139:P197" totalsRowShown="0">
+  <autoFilter ref="M139:P197" xr:uid="{826E6D02-7982-4253-94C2-5BA245328A25}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{6862BD12-4597-4214-B3EB-68C1564F73C6}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{66E5A46C-0B41-4BED-97A2-190992181AAE}" name="TALLA"/>
@@ -1822,8 +1850,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A26A5B85-3374-4A4B-B900-08F5F0C7C493}" name="Tabla41115163" displayName="Tabla41115163" ref="R135:U145" totalsRowShown="0">
-  <autoFilter ref="R135:U145" xr:uid="{A26A5B85-3374-4A4B-B900-08F5F0C7C493}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A26A5B85-3374-4A4B-B900-08F5F0C7C493}" name="Tabla41115163" displayName="Tabla41115163" ref="R139:U149" totalsRowShown="0">
+  <autoFilter ref="R139:U149" xr:uid="{A26A5B85-3374-4A4B-B900-08F5F0C7C493}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{BFD32BBC-DB8F-4DEA-95AE-1F3EFBCC6BCA}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{63FA53D9-9C6C-428E-AB82-456689F2A784}" name="TALLA"/>
@@ -1835,8 +1863,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{97430ED5-2D51-474D-AB3D-93DBD353FCE8}" name="Tabla4111516319" displayName="Tabla4111516319" ref="C151:F161" totalsRowShown="0">
-  <autoFilter ref="C151:F161" xr:uid="{97430ED5-2D51-474D-AB3D-93DBD353FCE8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{97430ED5-2D51-474D-AB3D-93DBD353FCE8}" name="Tabla4111516319" displayName="Tabla4111516319" ref="C155:F165" totalsRowShown="0">
+  <autoFilter ref="C155:F165" xr:uid="{97430ED5-2D51-474D-AB3D-93DBD353FCE8}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{D6BF6171-8DF6-440C-B202-55A2F70B2272}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{1CF84C6A-5C65-4163-9A2A-8F3288DF957D}" name="TALLA"/>
@@ -1848,8 +1876,8 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{1EE40C13-DCB7-4C11-84F8-663758F0A474}" name="Tabla411151631923" displayName="Tabla411151631923" ref="H135:K145" totalsRowShown="0">
-  <autoFilter ref="H135:K145" xr:uid="{1EE40C13-DCB7-4C11-84F8-663758F0A474}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{1EE40C13-DCB7-4C11-84F8-663758F0A474}" name="Tabla411151631923" displayName="Tabla411151631923" ref="H139:K149" totalsRowShown="0">
+  <autoFilter ref="H139:K149" xr:uid="{1EE40C13-DCB7-4C11-84F8-663758F0A474}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{567297BD-62AE-4B7A-A32B-93BAE1CEC9CF}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{3528AB60-B7F9-4600-AE95-46D8EA150570}" name="TALLA"/>
@@ -1861,8 +1889,8 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{155373F3-721B-42EA-A415-BA37094F5E9F}" name="Tabla411151636" displayName="Tabla411151636" ref="R151:U163" totalsRowShown="0">
-  <autoFilter ref="R151:U163" xr:uid="{155373F3-721B-42EA-A415-BA37094F5E9F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{155373F3-721B-42EA-A415-BA37094F5E9F}" name="Tabla411151636" displayName="Tabla411151636" ref="R155:U167" totalsRowShown="0">
+  <autoFilter ref="R155:U167" xr:uid="{155373F3-721B-42EA-A415-BA37094F5E9F}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{0CC4DA72-7CA1-4FC6-AF98-7D9117198F79}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{F08C3C9B-14B8-43D4-8CBC-0F877333A16B}" name="TALLA"/>
@@ -1874,8 +1902,8 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{46A5861F-102D-4F2D-9804-416AF2389DF2}" name="Tabla4111516367" displayName="Tabla4111516367" ref="R167:U177" totalsRowShown="0">
-  <autoFilter ref="R167:U177" xr:uid="{46A5861F-102D-4F2D-9804-416AF2389DF2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{46A5861F-102D-4F2D-9804-416AF2389DF2}" name="Tabla4111516367" displayName="Tabla4111516367" ref="R171:U181" totalsRowShown="0">
+  <autoFilter ref="R171:U181" xr:uid="{46A5861F-102D-4F2D-9804-416AF2389DF2}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{BFC964E9-7647-4AD2-B491-59C508B23244}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{39B6E5B8-BBF4-495B-9AA5-0F6BC4C39333}" name="TALLA"/>
@@ -1968,8 +1996,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{F5A69945-F316-48DA-AF9C-C495DB30FEB1}" name="Tabla4910" displayName="Tabla4910" ref="R5:U58" totalsRowShown="0">
-  <autoFilter ref="R5:U58" xr:uid="{F5A69945-F316-48DA-AF9C-C495DB30FEB1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{F5A69945-F316-48DA-AF9C-C495DB30FEB1}" name="Tabla4910" displayName="Tabla4910" ref="R5:U62" totalsRowShown="0">
+  <autoFilter ref="R5:U62" xr:uid="{F5A69945-F316-48DA-AF9C-C495DB30FEB1}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{FC68340A-34D4-46A4-B713-33E3D624245F}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{A31E3989-6B13-4AAD-ACF7-8DEA65F3D42E}" name="TALLA"/>
@@ -1981,8 +2009,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{94C85C53-33A5-44BD-B483-41B8989448CF}" name="Tabla411" displayName="Tabla411" ref="C62:F99" totalsRowShown="0">
-  <autoFilter ref="C62:F99" xr:uid="{94C85C53-33A5-44BD-B483-41B8989448CF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{94C85C53-33A5-44BD-B483-41B8989448CF}" name="Tabla411" displayName="Tabla411" ref="C66:F103" totalsRowShown="0">
+  <autoFilter ref="C66:F103" xr:uid="{94C85C53-33A5-44BD-B483-41B8989448CF}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{4D96F96D-BF60-49AE-9B75-BC6479C2EAEE}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{3080CCA9-BD26-4E0A-986F-CBE6D9C70A2D}" name="TALLA"/>
@@ -1994,8 +2022,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{4865AD5C-381F-47AF-8426-275903BA850B}" name="Tabla41112" displayName="Tabla41112" ref="H62:K132" totalsRowShown="0">
-  <autoFilter ref="H62:K132" xr:uid="{4865AD5C-381F-47AF-8426-275903BA850B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{4865AD5C-381F-47AF-8426-275903BA850B}" name="Tabla41112" displayName="Tabla41112" ref="H66:K136" totalsRowShown="0">
+  <autoFilter ref="H66:K136" xr:uid="{4865AD5C-381F-47AF-8426-275903BA850B}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{9508CA24-D2B9-49F8-B14E-E73D0C5D0324}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{7ECC0BAF-55A5-41D3-9865-AC4E8F0FE454}" name="TALLA"/>
@@ -2007,8 +2035,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{EC4F7B37-29F4-47EF-8F81-AF0F1C15CE63}" name="Tabla4111213" displayName="Tabla4111213" ref="M62:P72" totalsRowShown="0">
-  <autoFilter ref="M62:P72" xr:uid="{EC4F7B37-29F4-47EF-8F81-AF0F1C15CE63}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{EC4F7B37-29F4-47EF-8F81-AF0F1C15CE63}" name="Tabla4111213" displayName="Tabla4111213" ref="M66:P76" totalsRowShown="0">
+  <autoFilter ref="M66:P76" xr:uid="{EC4F7B37-29F4-47EF-8F81-AF0F1C15CE63}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{34455D18-34A3-46E3-9615-9D290C477AD6}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{F3DAEDA3-6B7A-4706-AA03-CFE2DDDE8428}" name="TALLA"/>
@@ -2020,8 +2048,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{188886CF-BAC4-4B7B-AADA-9EBECC49DE5B}" name="Tabla411121314" displayName="Tabla411121314" ref="R62:U84" totalsRowShown="0">
-  <autoFilter ref="R62:U84" xr:uid="{188886CF-BAC4-4B7B-AADA-9EBECC49DE5B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{188886CF-BAC4-4B7B-AADA-9EBECC49DE5B}" name="Tabla411121314" displayName="Tabla411121314" ref="R66:U88" totalsRowShown="0">
+  <autoFilter ref="R66:U88" xr:uid="{188886CF-BAC4-4B7B-AADA-9EBECC49DE5B}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{D24A1F41-57E3-4E13-BF9C-515D5619D263}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{EB0AE0B7-9DD8-42C5-A3C5-D039BD1EC8F7}" name="TALLA"/>
@@ -2033,8 +2061,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{410B3B57-302F-46A4-B190-E659B64689CC}" name="Tabla41115" displayName="Tabla41115" ref="C135:F145" totalsRowShown="0">
-  <autoFilter ref="C135:F145" xr:uid="{410B3B57-302F-46A4-B190-E659B64689CC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{410B3B57-302F-46A4-B190-E659B64689CC}" name="Tabla41115" displayName="Tabla41115" ref="C139:F149" totalsRowShown="0">
+  <autoFilter ref="C139:F149" xr:uid="{410B3B57-302F-46A4-B190-E659B64689CC}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{C40F20B7-FE80-4D54-9A49-8816ADEDD121}" name="CODIGO"/>
     <tableColumn id="2" xr3:uid="{E445583F-72EF-4D41-97F0-35356B18E440}" name="TALLA"/>
@@ -2342,7 +2370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FA982B6-DFA9-4840-9941-9DE0809894F7}">
-  <dimension ref="A4:U180"/>
+  <dimension ref="A4:U184"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
@@ -2364,30 +2392,30 @@
   </cols>
   <sheetData>
     <row r="4" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="H4" s="6" t="s">
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="H4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="M4" s="6" t="s">
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="M4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="R4" s="6" t="s">
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="R4" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="7"/>
+      <c r="U4" s="7"/>
     </row>
     <row r="5" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
@@ -3323,260 +3351,132 @@
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="R57" s="8" t="s">
+      <c r="R57" s="9" t="s">
         <v>486</v>
       </c>
-      <c r="S57" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="T57" s="8" t="s">
+      <c r="S57" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="T57" s="9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="R58" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="S58" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="T58" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="R59" t="s">
+        <v>496</v>
+      </c>
+      <c r="S59" t="s">
+        <v>4</v>
+      </c>
+      <c r="T59" t="s">
+        <v>497</v>
+      </c>
+    </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="C61" s="6" t="s">
+      <c r="A61" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="64" spans="1:21" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C65" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D61" s="6"/>
-      <c r="E61" s="6"/>
-      <c r="F61" s="6"/>
-      <c r="H61" s="6" t="s">
+      <c r="D65" s="7"/>
+      <c r="E65" s="7"/>
+      <c r="F65" s="7"/>
+      <c r="H65" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I61" s="6"/>
-      <c r="J61" s="6"/>
-      <c r="K61" s="6"/>
-      <c r="M61" s="6" t="s">
+      <c r="I65" s="7"/>
+      <c r="J65" s="7"/>
+      <c r="K65" s="7"/>
+      <c r="M65" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="N61" s="6"/>
-      <c r="O61" s="6"/>
-      <c r="P61" s="6"/>
-      <c r="R61" s="6" t="s">
+      <c r="N65" s="7"/>
+      <c r="O65" s="7"/>
+      <c r="P65" s="7"/>
+      <c r="R65" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="S61" s="6"/>
-      <c r="T61" s="6"/>
-      <c r="U61" s="6"/>
-    </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="C62" t="s">
+      <c r="S65" s="7"/>
+      <c r="T65" s="7"/>
+      <c r="U65" s="7"/>
+    </row>
+    <row r="66" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C66" t="s">
         <v>2</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D66" t="s">
         <v>3</v>
       </c>
-      <c r="E62" t="s">
+      <c r="E66" t="s">
         <v>6</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F66" t="s">
         <v>86</v>
       </c>
-      <c r="H62" t="s">
+      <c r="H66" t="s">
         <v>2</v>
       </c>
-      <c r="I62" t="s">
+      <c r="I66" t="s">
         <v>3</v>
       </c>
-      <c r="J62" t="s">
+      <c r="J66" t="s">
         <v>6</v>
       </c>
-      <c r="K62" t="s">
+      <c r="K66" t="s">
         <v>86</v>
       </c>
-      <c r="M62" t="s">
+      <c r="M66" t="s">
         <v>2</v>
       </c>
-      <c r="N62" t="s">
+      <c r="N66" t="s">
         <v>3</v>
       </c>
-      <c r="O62" t="s">
+      <c r="O66" t="s">
         <v>6</v>
       </c>
-      <c r="P62" t="s">
+      <c r="P66" t="s">
         <v>86</v>
       </c>
-      <c r="R62" t="s">
+      <c r="R66" t="s">
         <v>2</v>
       </c>
-      <c r="S62" t="s">
+      <c r="S66" t="s">
         <v>3</v>
       </c>
-      <c r="T62" t="s">
+      <c r="T66" t="s">
         <v>6</v>
       </c>
-      <c r="U62" t="s">
+      <c r="U66" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="C63" t="s">
+    <row r="67" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C67" t="s">
         <v>26</v>
       </c>
-      <c r="D63" t="s">
+      <c r="D67" t="s">
         <v>10</v>
       </c>
-      <c r="E63" t="s">
+      <c r="E67" t="s">
         <v>23</v>
       </c>
-      <c r="H63" t="s">
+      <c r="H67" t="s">
         <v>30</v>
-      </c>
-      <c r="I63" t="s">
-        <v>18</v>
-      </c>
-      <c r="J63" t="s">
-        <v>7</v>
-      </c>
-      <c r="M63" t="s">
-        <v>32</v>
-      </c>
-      <c r="N63" t="s">
-        <v>1</v>
-      </c>
-      <c r="O63" t="s">
-        <v>13</v>
-      </c>
-      <c r="R63" t="s">
-        <v>37</v>
-      </c>
-      <c r="S63" t="s">
-        <v>1</v>
-      </c>
-      <c r="T63" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="C64" t="s">
-        <v>27</v>
-      </c>
-      <c r="D64" t="s">
-        <v>18</v>
-      </c>
-      <c r="E64" t="s">
-        <v>7</v>
-      </c>
-      <c r="H64" t="s">
-        <v>42</v>
-      </c>
-      <c r="I64" t="s">
-        <v>10</v>
-      </c>
-      <c r="J64" t="s">
-        <v>7</v>
-      </c>
-      <c r="M64" t="s">
-        <v>53</v>
-      </c>
-      <c r="N64" t="s">
-        <v>10</v>
-      </c>
-      <c r="O64" t="s">
-        <v>13</v>
-      </c>
-      <c r="R64" t="s">
-        <v>38</v>
-      </c>
-      <c r="S64" t="s">
-        <v>4</v>
-      </c>
-      <c r="T64" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="65" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C65" t="s">
-        <v>28</v>
-      </c>
-      <c r="D65" t="s">
-        <v>1</v>
-      </c>
-      <c r="E65" t="s">
-        <v>29</v>
-      </c>
-      <c r="H65" t="s">
-        <v>47</v>
-      </c>
-      <c r="I65" t="s">
-        <v>10</v>
-      </c>
-      <c r="J65" t="s">
-        <v>398</v>
-      </c>
-      <c r="M65" t="s">
-        <v>70</v>
-      </c>
-      <c r="N65" t="s">
-        <v>18</v>
-      </c>
-      <c r="O65" t="s">
-        <v>71</v>
-      </c>
-      <c r="R65" t="s">
-        <v>57</v>
-      </c>
-      <c r="S65" t="s">
-        <v>18</v>
-      </c>
-      <c r="T65" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="66" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C66" t="s">
-        <v>54</v>
-      </c>
-      <c r="D66" t="s">
-        <v>10</v>
-      </c>
-      <c r="E66" t="s">
-        <v>13</v>
-      </c>
-      <c r="H66" t="s">
-        <v>49</v>
-      </c>
-      <c r="I66" t="s">
-        <v>18</v>
-      </c>
-      <c r="J66" t="s">
-        <v>48</v>
-      </c>
-      <c r="M66" t="s">
-        <v>79</v>
-      </c>
-      <c r="N66" t="s">
-        <v>10</v>
-      </c>
-      <c r="O66" t="s">
-        <v>13</v>
-      </c>
-      <c r="P66" t="s">
-        <v>115</v>
-      </c>
-      <c r="R66" t="s">
-        <v>58</v>
-      </c>
-      <c r="S66" t="s">
-        <v>4</v>
-      </c>
-      <c r="T66" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="67" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C67" t="s">
-        <v>286</v>
-      </c>
-      <c r="D67" t="s">
-        <v>18</v>
-      </c>
-      <c r="E67" t="s">
-        <v>46</v>
-      </c>
-      <c r="H67" t="s">
-        <v>50</v>
       </c>
       <c r="I67" t="s">
         <v>18</v>
@@ -3585,621 +3485,759 @@
         <v>7</v>
       </c>
       <c r="M67" t="s">
-        <v>81</v>
+        <v>32</v>
       </c>
       <c r="N67" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O67" t="s">
         <v>13</v>
       </c>
       <c r="R67" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="S67" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="T67" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="68" spans="3:20" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="68" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C68" t="s">
-        <v>287</v>
+        <v>27</v>
       </c>
       <c r="D68" t="s">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E68" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="H68" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="I68" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J68" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="M68" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="N68" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="O68" t="s">
         <v>13</v>
       </c>
-      <c r="P68" t="s">
-        <v>115</v>
-      </c>
       <c r="R68" t="s">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="S68" t="s">
         <v>4</v>
       </c>
       <c r="T68" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="69" spans="3:20" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="69" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C69" t="s">
-        <v>288</v>
+        <v>28</v>
       </c>
       <c r="D69" t="s">
-        <v>302</v>
+        <v>1</v>
       </c>
       <c r="E69" t="s">
-        <v>303</v>
+        <v>29</v>
       </c>
       <c r="H69" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
       <c r="I69" t="s">
-        <v>424</v>
+        <v>10</v>
       </c>
       <c r="J69" t="s">
-        <v>124</v>
+        <v>398</v>
       </c>
       <c r="M69" t="s">
-        <v>374</v>
+        <v>70</v>
       </c>
       <c r="N69" t="s">
         <v>18</v>
       </c>
       <c r="O69" t="s">
+        <v>71</v>
+      </c>
+      <c r="R69" t="s">
+        <v>57</v>
+      </c>
+      <c r="S69" t="s">
+        <v>18</v>
+      </c>
+      <c r="T69" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="70" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C70" t="s">
+        <v>54</v>
+      </c>
+      <c r="D70" t="s">
+        <v>10</v>
+      </c>
+      <c r="E70" t="s">
         <v>13</v>
       </c>
-      <c r="P69" t="s">
-        <v>115</v>
-      </c>
-      <c r="R69" t="s">
-        <v>75</v>
-      </c>
-      <c r="S69" t="s">
-        <v>4</v>
-      </c>
-      <c r="T69" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="70" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C70" t="s">
-        <v>289</v>
-      </c>
-      <c r="D70" t="s">
-        <v>123</v>
-      </c>
-      <c r="E70" t="s">
-        <v>7</v>
-      </c>
       <c r="H70" t="s">
-        <v>151</v>
+        <v>49</v>
       </c>
       <c r="I70" t="s">
+        <v>18</v>
+      </c>
+      <c r="J70" t="s">
+        <v>48</v>
+      </c>
+      <c r="M70" t="s">
+        <v>79</v>
+      </c>
+      <c r="N70" t="s">
         <v>10</v>
-      </c>
-      <c r="J70" t="s">
-        <v>107</v>
-      </c>
-      <c r="M70" t="s">
-        <v>404</v>
-      </c>
-      <c r="N70" t="s">
-        <v>1</v>
       </c>
       <c r="O70" t="s">
         <v>13</v>
       </c>
+      <c r="P70" t="s">
+        <v>115</v>
+      </c>
       <c r="R70" t="s">
+        <v>58</v>
+      </c>
+      <c r="S70" t="s">
+        <v>4</v>
+      </c>
+      <c r="T70" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="71" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C71" t="s">
+        <v>286</v>
+      </c>
+      <c r="D71" t="s">
+        <v>18</v>
+      </c>
+      <c r="E71" t="s">
+        <v>46</v>
+      </c>
+      <c r="H71" t="s">
+        <v>50</v>
+      </c>
+      <c r="I71" t="s">
+        <v>18</v>
+      </c>
+      <c r="J71" t="s">
+        <v>7</v>
+      </c>
+      <c r="M71" t="s">
+        <v>81</v>
+      </c>
+      <c r="N71" t="s">
+        <v>10</v>
+      </c>
+      <c r="O71" t="s">
+        <v>13</v>
+      </c>
+      <c r="R71" t="s">
+        <v>68</v>
+      </c>
+      <c r="S71" t="s">
+        <v>18</v>
+      </c>
+      <c r="T71" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="72" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C72" t="s">
+        <v>287</v>
+      </c>
+      <c r="D72" t="s">
+        <v>1</v>
+      </c>
+      <c r="E72" t="s">
+        <v>48</v>
+      </c>
+      <c r="H72" t="s">
+        <v>59</v>
+      </c>
+      <c r="I72" t="s">
+        <v>4</v>
+      </c>
+      <c r="J72" t="s">
+        <v>13</v>
+      </c>
+      <c r="M72" t="s">
+        <v>85</v>
+      </c>
+      <c r="N72" t="s">
+        <v>1</v>
+      </c>
+      <c r="O72" t="s">
+        <v>13</v>
+      </c>
+      <c r="P72" t="s">
+        <v>115</v>
+      </c>
+      <c r="R72" t="s">
+        <v>72</v>
+      </c>
+      <c r="S72" t="s">
+        <v>4</v>
+      </c>
+      <c r="T72" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="73" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C73" t="s">
+        <v>288</v>
+      </c>
+      <c r="D73" t="s">
+        <v>302</v>
+      </c>
+      <c r="E73" t="s">
+        <v>303</v>
+      </c>
+      <c r="H73" t="s">
+        <v>122</v>
+      </c>
+      <c r="I73" t="s">
+        <v>424</v>
+      </c>
+      <c r="J73" t="s">
+        <v>124</v>
+      </c>
+      <c r="M73" t="s">
+        <v>374</v>
+      </c>
+      <c r="N73" t="s">
+        <v>18</v>
+      </c>
+      <c r="O73" t="s">
+        <v>13</v>
+      </c>
+      <c r="P73" t="s">
+        <v>115</v>
+      </c>
+      <c r="R73" t="s">
+        <v>75</v>
+      </c>
+      <c r="S73" t="s">
+        <v>4</v>
+      </c>
+      <c r="T73" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="74" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C74" t="s">
+        <v>289</v>
+      </c>
+      <c r="D74" t="s">
+        <v>123</v>
+      </c>
+      <c r="E74" t="s">
+        <v>7</v>
+      </c>
+      <c r="H74" t="s">
+        <v>151</v>
+      </c>
+      <c r="I74" t="s">
+        <v>10</v>
+      </c>
+      <c r="J74" t="s">
+        <v>107</v>
+      </c>
+      <c r="M74" t="s">
+        <v>404</v>
+      </c>
+      <c r="N74" t="s">
+        <v>1</v>
+      </c>
+      <c r="O74" t="s">
+        <v>13</v>
+      </c>
+      <c r="R74" t="s">
         <v>83</v>
       </c>
-      <c r="S70" t="s">
+      <c r="S74" t="s">
         <v>10</v>
       </c>
-      <c r="T70" t="s">
+      <c r="T74" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C71" t="s">
+    <row r="75" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C75" t="s">
         <v>290</v>
       </c>
-      <c r="D71" t="s">
+      <c r="D75" t="s">
         <v>10</v>
-      </c>
-      <c r="E71" t="s">
-        <v>94</v>
-      </c>
-      <c r="H71" t="s">
-        <v>165</v>
-      </c>
-      <c r="I71" t="s">
-        <v>4</v>
-      </c>
-      <c r="J71" t="s">
-        <v>13</v>
-      </c>
-      <c r="R71" t="s">
-        <v>314</v>
-      </c>
-      <c r="S71" t="s">
-        <v>4</v>
-      </c>
-      <c r="T71" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="72" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C72" t="s">
-        <v>291</v>
-      </c>
-      <c r="D72" t="s">
-        <v>18</v>
-      </c>
-      <c r="E72" t="s">
-        <v>304</v>
-      </c>
-      <c r="H72" t="s">
-        <v>175</v>
-      </c>
-      <c r="I72" t="s">
-        <v>18</v>
-      </c>
-      <c r="J72" t="s">
-        <v>176</v>
-      </c>
-      <c r="R72" t="s">
-        <v>316</v>
-      </c>
-      <c r="S72" t="s">
-        <v>4</v>
-      </c>
-      <c r="T72" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="73" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C73" t="s">
-        <v>292</v>
-      </c>
-      <c r="D73" t="s">
-        <v>18</v>
-      </c>
-      <c r="E73" t="s">
-        <v>236</v>
-      </c>
-      <c r="H73" t="s">
-        <v>177</v>
-      </c>
-      <c r="I73" t="s">
-        <v>18</v>
-      </c>
-      <c r="J73" t="s">
-        <v>13</v>
-      </c>
-      <c r="R73" t="s">
-        <v>317</v>
-      </c>
-      <c r="S73" t="s">
-        <v>1</v>
-      </c>
-      <c r="T73" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="74" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C74" t="s">
-        <v>293</v>
-      </c>
-      <c r="D74" t="s">
-        <v>18</v>
-      </c>
-      <c r="E74" t="s">
-        <v>13</v>
-      </c>
-      <c r="H74" t="s">
-        <v>192</v>
-      </c>
-      <c r="I74" t="s">
-        <v>18</v>
-      </c>
-      <c r="J74" t="s">
-        <v>13</v>
-      </c>
-      <c r="R74" t="s">
-        <v>318</v>
-      </c>
-      <c r="S74" t="s">
-        <v>20</v>
-      </c>
-      <c r="T74" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="75" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C75" t="s">
-        <v>294</v>
-      </c>
-      <c r="D75" t="s">
-        <v>18</v>
       </c>
       <c r="E75" t="s">
         <v>94</v>
       </c>
       <c r="H75" t="s">
+        <v>165</v>
+      </c>
+      <c r="I75" t="s">
+        <v>4</v>
+      </c>
+      <c r="J75" t="s">
+        <v>13</v>
+      </c>
+      <c r="R75" t="s">
+        <v>314</v>
+      </c>
+      <c r="S75" t="s">
+        <v>4</v>
+      </c>
+      <c r="T75" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="76" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C76" t="s">
+        <v>291</v>
+      </c>
+      <c r="D76" t="s">
+        <v>18</v>
+      </c>
+      <c r="E76" t="s">
+        <v>304</v>
+      </c>
+      <c r="H76" t="s">
+        <v>175</v>
+      </c>
+      <c r="I76" t="s">
+        <v>18</v>
+      </c>
+      <c r="J76" t="s">
+        <v>176</v>
+      </c>
+      <c r="R76" t="s">
+        <v>316</v>
+      </c>
+      <c r="S76" t="s">
+        <v>4</v>
+      </c>
+      <c r="T76" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="77" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C77" t="s">
+        <v>292</v>
+      </c>
+      <c r="D77" t="s">
+        <v>18</v>
+      </c>
+      <c r="E77" t="s">
+        <v>236</v>
+      </c>
+      <c r="H77" t="s">
+        <v>177</v>
+      </c>
+      <c r="I77" t="s">
+        <v>18</v>
+      </c>
+      <c r="J77" t="s">
+        <v>13</v>
+      </c>
+      <c r="R77" t="s">
+        <v>317</v>
+      </c>
+      <c r="S77" t="s">
+        <v>1</v>
+      </c>
+      <c r="T77" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="78" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C78" t="s">
+        <v>293</v>
+      </c>
+      <c r="D78" t="s">
+        <v>18</v>
+      </c>
+      <c r="E78" t="s">
+        <v>13</v>
+      </c>
+      <c r="H78" t="s">
+        <v>192</v>
+      </c>
+      <c r="I78" t="s">
+        <v>18</v>
+      </c>
+      <c r="J78" t="s">
+        <v>13</v>
+      </c>
+      <c r="R78" t="s">
+        <v>318</v>
+      </c>
+      <c r="S78" t="s">
+        <v>20</v>
+      </c>
+      <c r="T78" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="79" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C79" t="s">
+        <v>294</v>
+      </c>
+      <c r="D79" t="s">
+        <v>18</v>
+      </c>
+      <c r="E79" t="s">
+        <v>94</v>
+      </c>
+      <c r="H79" t="s">
         <v>193</v>
       </c>
-      <c r="I75" t="s">
-        <v>18</v>
-      </c>
-      <c r="J75" t="s">
+      <c r="I79" t="s">
+        <v>18</v>
+      </c>
+      <c r="J79" t="s">
         <v>7</v>
       </c>
-      <c r="R75" t="s">
+      <c r="R79" t="s">
         <v>319</v>
       </c>
-      <c r="S75" t="s">
-        <v>18</v>
-      </c>
-      <c r="T75" t="s">
+      <c r="S79" t="s">
+        <v>18</v>
+      </c>
+      <c r="T79" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="76" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C76" t="s">
+    <row r="80" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C80" t="s">
         <v>295</v>
-      </c>
-      <c r="D76" t="s">
-        <v>20</v>
-      </c>
-      <c r="E76" t="s">
-        <v>13</v>
-      </c>
-      <c r="H76" t="s">
-        <v>194</v>
-      </c>
-      <c r="I76" t="s">
-        <v>18</v>
-      </c>
-      <c r="J76" t="s">
-        <v>202</v>
-      </c>
-      <c r="R76" t="s">
-        <v>320</v>
-      </c>
-      <c r="S76" t="s">
-        <v>20</v>
-      </c>
-      <c r="T76" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="77" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C77" t="s">
-        <v>296</v>
-      </c>
-      <c r="D77" t="s">
-        <v>1</v>
-      </c>
-      <c r="E77" t="s">
-        <v>7</v>
-      </c>
-      <c r="H77" t="s">
-        <v>195</v>
-      </c>
-      <c r="I77" t="s">
-        <v>18</v>
-      </c>
-      <c r="J77" t="s">
-        <v>46</v>
-      </c>
-      <c r="R77" t="s">
-        <v>321</v>
-      </c>
-      <c r="S77" t="s">
-        <v>4</v>
-      </c>
-      <c r="T77" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="78" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C78" t="s">
-        <v>297</v>
-      </c>
-      <c r="D78" t="s">
-        <v>18</v>
-      </c>
-      <c r="E78" t="s">
-        <v>305</v>
-      </c>
-      <c r="H78" t="s">
-        <v>196</v>
-      </c>
-      <c r="I78" t="s">
-        <v>18</v>
-      </c>
-      <c r="J78" t="s">
-        <v>171</v>
-      </c>
-      <c r="R78" t="s">
-        <v>323</v>
-      </c>
-      <c r="S78" t="s">
-        <v>18</v>
-      </c>
-      <c r="T78" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="79" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C79" t="s">
-        <v>298</v>
-      </c>
-      <c r="D79" t="s">
-        <v>1</v>
-      </c>
-      <c r="E79" t="s">
-        <v>13</v>
-      </c>
-      <c r="H79" t="s">
-        <v>197</v>
-      </c>
-      <c r="I79" t="s">
-        <v>18</v>
-      </c>
-      <c r="J79" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="80" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C80" t="s">
-        <v>299</v>
       </c>
       <c r="D80" t="s">
         <v>20</v>
       </c>
       <c r="E80" t="s">
+        <v>13</v>
+      </c>
+      <c r="H80" t="s">
+        <v>194</v>
+      </c>
+      <c r="I80" t="s">
+        <v>18</v>
+      </c>
+      <c r="J80" t="s">
+        <v>202</v>
+      </c>
+      <c r="R80" t="s">
+        <v>320</v>
+      </c>
+      <c r="S80" t="s">
+        <v>20</v>
+      </c>
+      <c r="T80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="C81" t="s">
+        <v>296</v>
+      </c>
+      <c r="D81" t="s">
+        <v>1</v>
+      </c>
+      <c r="E81" t="s">
         <v>7</v>
       </c>
-      <c r="H80" t="s">
+      <c r="H81" t="s">
+        <v>195</v>
+      </c>
+      <c r="I81" t="s">
+        <v>18</v>
+      </c>
+      <c r="J81" t="s">
+        <v>46</v>
+      </c>
+      <c r="R81" t="s">
+        <v>321</v>
+      </c>
+      <c r="S81" t="s">
+        <v>4</v>
+      </c>
+      <c r="T81" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="82" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="C82" t="s">
+        <v>297</v>
+      </c>
+      <c r="D82" t="s">
+        <v>18</v>
+      </c>
+      <c r="E82" t="s">
+        <v>305</v>
+      </c>
+      <c r="H82" t="s">
+        <v>196</v>
+      </c>
+      <c r="I82" t="s">
+        <v>18</v>
+      </c>
+      <c r="J82" t="s">
+        <v>171</v>
+      </c>
+      <c r="R82" t="s">
+        <v>323</v>
+      </c>
+      <c r="S82" t="s">
+        <v>18</v>
+      </c>
+      <c r="T82" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="83" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="C83" t="s">
+        <v>298</v>
+      </c>
+      <c r="D83" t="s">
+        <v>1</v>
+      </c>
+      <c r="E83" t="s">
+        <v>13</v>
+      </c>
+      <c r="H83" t="s">
+        <v>197</v>
+      </c>
+      <c r="I83" t="s">
+        <v>18</v>
+      </c>
+      <c r="J83" t="s">
+        <v>13</v>
+      </c>
+      <c r="R83" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="S83" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="T83" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="84" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="C84" t="s">
+        <v>299</v>
+      </c>
+      <c r="D84" t="s">
+        <v>20</v>
+      </c>
+      <c r="E84" t="s">
+        <v>7</v>
+      </c>
+      <c r="H84" t="s">
         <v>198</v>
       </c>
-      <c r="I80" t="s">
-        <v>18</v>
-      </c>
-      <c r="J80" t="s">
+      <c r="I84" t="s">
+        <v>18</v>
+      </c>
+      <c r="J84" t="s">
         <v>203</v>
       </c>
-      <c r="N80" s="1"/>
-    </row>
-    <row r="81" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C81" t="s">
+      <c r="N84" s="1"/>
+    </row>
+    <row r="85" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="C85" t="s">
         <v>300</v>
       </c>
-      <c r="D81" t="s">
-        <v>4</v>
-      </c>
-      <c r="E81" t="s">
+      <c r="D85" t="s">
+        <v>4</v>
+      </c>
+      <c r="E85" t="s">
         <v>94</v>
       </c>
-      <c r="H81" t="s">
+      <c r="H85" t="s">
         <v>199</v>
       </c>
-      <c r="I81" t="s">
-        <v>18</v>
-      </c>
-      <c r="J81" t="s">
+      <c r="I85" t="s">
+        <v>18</v>
+      </c>
+      <c r="J85" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="82" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C82" t="s">
+    <row r="86" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="C86" t="s">
         <v>301</v>
       </c>
-      <c r="D82" t="s">
+      <c r="D86" t="s">
         <v>307</v>
       </c>
-      <c r="E82" t="s">
+      <c r="E86" t="s">
         <v>306</v>
       </c>
-      <c r="H82" t="s">
+      <c r="H86" t="s">
         <v>200</v>
-      </c>
-      <c r="I82" t="s">
-        <v>1</v>
-      </c>
-      <c r="J82" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="83" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C83" t="s">
-        <v>475</v>
-      </c>
-      <c r="D83" t="s">
-        <v>18</v>
-      </c>
-      <c r="E83" t="s">
-        <v>476</v>
-      </c>
-      <c r="H83" t="s">
-        <v>201</v>
-      </c>
-      <c r="I83" t="s">
-        <v>4</v>
-      </c>
-      <c r="J83" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="84" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="H84" t="s">
-        <v>204</v>
-      </c>
-      <c r="I84" t="s">
-        <v>4</v>
-      </c>
-      <c r="J84" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="85" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="H85" t="s">
-        <v>205</v>
-      </c>
-      <c r="I85" t="s">
-        <v>1</v>
-      </c>
-      <c r="J85" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="86" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="H86" t="s">
-        <v>206</v>
       </c>
       <c r="I86" t="s">
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="87" spans="3:11" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="87" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="C87" t="s">
+        <v>475</v>
+      </c>
+      <c r="D87" t="s">
+        <v>18</v>
+      </c>
+      <c r="E87" t="s">
+        <v>476</v>
+      </c>
       <c r="H87" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="I87" t="s">
+        <v>4</v>
+      </c>
+      <c r="J87" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="88" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="C88" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="H88" t="s">
+        <v>204</v>
+      </c>
+      <c r="I88" t="s">
+        <v>4</v>
+      </c>
+      <c r="J88" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="89" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="C89" t="s">
+        <v>495</v>
+      </c>
+      <c r="D89" t="s">
         <v>1</v>
       </c>
-      <c r="J87" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="88" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="H88" t="s">
-        <v>208</v>
-      </c>
-      <c r="I88" t="s">
-        <v>1</v>
-      </c>
-      <c r="J88" t="s">
-        <v>7</v>
-      </c>
-      <c r="K88" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="89" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E89" t="s">
+        <v>23</v>
+      </c>
       <c r="H89" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="I89" t="s">
         <v>1</v>
       </c>
       <c r="J89" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="90" spans="3:11" x14ac:dyDescent="0.25">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="90" spans="3:20" x14ac:dyDescent="0.25">
       <c r="H90" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="I90" t="s">
         <v>1</v>
       </c>
       <c r="J90" t="s">
-        <v>48</v>
-      </c>
-      <c r="K90" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="91" spans="3:11" x14ac:dyDescent="0.25">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="91" spans="3:20" x14ac:dyDescent="0.25">
       <c r="H91" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="I91" t="s">
         <v>1</v>
       </c>
       <c r="J91" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="92" spans="3:11" x14ac:dyDescent="0.25">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="92" spans="3:20" x14ac:dyDescent="0.25">
       <c r="H92" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="I92" t="s">
         <v>1</v>
       </c>
       <c r="J92" t="s">
+        <v>7</v>
+      </c>
+      <c r="K92" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="93" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="H93" t="s">
+        <v>209</v>
+      </c>
+      <c r="I93" t="s">
+        <v>1</v>
+      </c>
+      <c r="J93" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="94" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="H94" t="s">
+        <v>210</v>
+      </c>
+      <c r="I94" t="s">
+        <v>1</v>
+      </c>
+      <c r="J94" t="s">
+        <v>48</v>
+      </c>
+      <c r="K94" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="95" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="H95" t="s">
+        <v>211</v>
+      </c>
+      <c r="I95" t="s">
+        <v>1</v>
+      </c>
+      <c r="J95" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="93" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="H93" t="s">
-        <v>216</v>
-      </c>
-      <c r="I93" t="s">
-        <v>10</v>
-      </c>
-      <c r="J93" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="94" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="H94" t="s">
-        <v>217</v>
-      </c>
-      <c r="I94" t="s">
-        <v>4</v>
-      </c>
-      <c r="J94" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="95" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="H95" t="s">
-        <v>218</v>
-      </c>
-      <c r="I95" t="s">
-        <v>20</v>
-      </c>
-      <c r="J95" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="96" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="96" spans="3:20" x14ac:dyDescent="0.25">
       <c r="H96" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="I96" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J96" t="s">
         <v>13</v>
@@ -4207,7 +4245,7 @@
     </row>
     <row r="97" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H97" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="I97" t="s">
         <v>10</v>
@@ -4218,134 +4256,134 @@
     </row>
     <row r="98" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H98" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="I98" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J98" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
     </row>
     <row r="99" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H99" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="I99" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J99" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="100" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H100" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="I100" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J100" t="s">
-        <v>226</v>
+        <v>13</v>
       </c>
     </row>
     <row r="101" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H101" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="I101" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J101" t="s">
-        <v>285</v>
-      </c>
-      <c r="K101" t="s">
-        <v>115</v>
+        <v>13</v>
       </c>
     </row>
     <row r="102" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H102" t="s">
-        <v>308</v>
+        <v>221</v>
       </c>
       <c r="I102" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="J102" t="s">
-        <v>309</v>
+        <v>224</v>
       </c>
     </row>
     <row r="103" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H103" t="s">
-        <v>310</v>
+        <v>222</v>
       </c>
       <c r="I103" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="J103" t="s">
-        <v>13</v>
+        <v>225</v>
       </c>
     </row>
     <row r="104" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H104" t="s">
-        <v>311</v>
+        <v>227</v>
       </c>
       <c r="I104" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J104" t="s">
-        <v>7</v>
+        <v>226</v>
       </c>
     </row>
     <row r="105" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H105" t="s">
-        <v>428</v>
+        <v>228</v>
       </c>
       <c r="I105" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="J105" t="s">
-        <v>7</v>
+        <v>285</v>
+      </c>
+      <c r="K105" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="106" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H106" t="s">
-        <v>429</v>
+        <v>308</v>
       </c>
       <c r="I106" t="s">
         <v>18</v>
       </c>
       <c r="J106" t="s">
-        <v>13</v>
+        <v>309</v>
       </c>
     </row>
     <row r="107" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H107" t="s">
-        <v>430</v>
+        <v>310</v>
       </c>
       <c r="I107" t="s">
         <v>18</v>
       </c>
       <c r="J107" t="s">
-        <v>431</v>
+        <v>13</v>
       </c>
     </row>
     <row r="108" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H108" t="s">
-        <v>432</v>
+        <v>311</v>
       </c>
       <c r="I108" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J108" t="s">
-        <v>107</v>
+        <v>7</v>
       </c>
     </row>
     <row r="109" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H109" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="I109" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="J109" t="s">
         <v>7</v>
@@ -4353,1581 +4391,1637 @@
     </row>
     <row r="110" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H110" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="I110" t="s">
-        <v>435</v>
+        <v>18</v>
       </c>
       <c r="J110" t="s">
-        <v>332</v>
+        <v>13</v>
       </c>
     </row>
     <row r="111" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H111" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="I111" t="s">
-        <v>435</v>
+        <v>18</v>
       </c>
       <c r="J111" t="s">
-        <v>422</v>
+        <v>431</v>
       </c>
     </row>
     <row r="112" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H112" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="I112" t="s">
-        <v>438</v>
+        <v>10</v>
       </c>
       <c r="J112" t="s">
-        <v>332</v>
+        <v>107</v>
       </c>
     </row>
     <row r="113" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H113" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
       <c r="I113" t="s">
-        <v>435</v>
+        <v>4</v>
       </c>
       <c r="J113" t="s">
-        <v>440</v>
+        <v>7</v>
       </c>
     </row>
     <row r="114" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H114" t="s">
-        <v>441</v>
+        <v>434</v>
       </c>
       <c r="I114" t="s">
-        <v>424</v>
+        <v>435</v>
       </c>
       <c r="J114" t="s">
-        <v>442</v>
+        <v>332</v>
       </c>
     </row>
     <row r="115" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H115" t="s">
-        <v>443</v>
+        <v>436</v>
       </c>
       <c r="I115" t="s">
-        <v>424</v>
+        <v>435</v>
       </c>
       <c r="J115" t="s">
-        <v>444</v>
+        <v>422</v>
       </c>
     </row>
     <row r="116" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H116" t="s">
-        <v>449</v>
+        <v>437</v>
       </c>
       <c r="I116" t="s">
-        <v>424</v>
+        <v>438</v>
       </c>
       <c r="J116" t="s">
-        <v>450</v>
+        <v>332</v>
       </c>
     </row>
     <row r="117" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H117" t="s">
-        <v>451</v>
+        <v>439</v>
       </c>
       <c r="I117" t="s">
-        <v>424</v>
+        <v>435</v>
       </c>
       <c r="J117" t="s">
-        <v>7</v>
+        <v>440</v>
       </c>
     </row>
     <row r="118" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H118" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="I118" t="s">
         <v>424</v>
       </c>
       <c r="J118" t="s">
-        <v>29</v>
+        <v>442</v>
       </c>
     </row>
     <row r="119" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H119" t="s">
-        <v>453</v>
+        <v>443</v>
       </c>
       <c r="I119" t="s">
-        <v>1</v>
+        <v>424</v>
       </c>
       <c r="J119" t="s">
-        <v>454</v>
+        <v>444</v>
       </c>
     </row>
     <row r="120" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H120" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="I120" t="s">
-        <v>4</v>
+        <v>424</v>
       </c>
       <c r="J120" t="s">
-        <v>7</v>
+        <v>450</v>
       </c>
     </row>
     <row r="121" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H121" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="I121" t="s">
-        <v>1</v>
+        <v>424</v>
       </c>
       <c r="J121" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="122" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H122" t="s">
-        <v>463</v>
+        <v>452</v>
       </c>
       <c r="I122" t="s">
-        <v>10</v>
+        <v>424</v>
       </c>
       <c r="J122" t="s">
-        <v>124</v>
+        <v>29</v>
       </c>
     </row>
     <row r="123" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H123" t="s">
-        <v>465</v>
+        <v>453</v>
       </c>
       <c r="I123" t="s">
-        <v>466</v>
+        <v>1</v>
       </c>
       <c r="J123" t="s">
-        <v>467</v>
+        <v>454</v>
       </c>
     </row>
     <row r="124" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H124" t="s">
-        <v>468</v>
+        <v>455</v>
       </c>
       <c r="I124" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J124" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H125" t="s">
-        <v>469</v>
+        <v>456</v>
       </c>
       <c r="I125" t="s">
+        <v>1</v>
+      </c>
+      <c r="J125" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="126" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H126" t="s">
+        <v>463</v>
+      </c>
+      <c r="I126" t="s">
         <v>10</v>
       </c>
-      <c r="J125" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="126" spans="8:10" x14ac:dyDescent="0.25">
-      <c r="H126" s="8" t="s">
-        <v>477</v>
-      </c>
-      <c r="I126" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="J126" s="8" t="s">
-        <v>13</v>
+      <c r="J126" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="127" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H127" t="s">
-        <v>478</v>
+        <v>465</v>
       </c>
       <c r="I127" t="s">
-        <v>1</v>
+        <v>466</v>
       </c>
       <c r="J127" t="s">
-        <v>9</v>
+        <v>467</v>
       </c>
     </row>
     <row r="128" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H128" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="I128" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="J128" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="129" spans="3:21" x14ac:dyDescent="0.25">
       <c r="H129" t="s">
+        <v>469</v>
+      </c>
+      <c r="I129" t="s">
+        <v>10</v>
+      </c>
+      <c r="J129" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="130" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H130" s="9" t="s">
+        <v>477</v>
+      </c>
+      <c r="I130" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="J130" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="131" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H131" t="s">
+        <v>478</v>
+      </c>
+      <c r="I131" t="s">
+        <v>1</v>
+      </c>
+      <c r="J131" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="132" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H132" t="s">
+        <v>487</v>
+      </c>
+      <c r="I132" t="s">
+        <v>18</v>
+      </c>
+      <c r="J132" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="133" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H133" t="s">
         <v>488</v>
       </c>
-      <c r="I129" t="s">
+      <c r="I133" t="s">
         <v>1</v>
       </c>
-      <c r="J129" t="s">
+      <c r="J133" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="134" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C134" s="6" t="s">
+      <c r="H134" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="I134" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J134" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="K134" s="6"/>
+    </row>
+    <row r="138" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C138" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D134" s="6"/>
-      <c r="E134" s="6"/>
-      <c r="F134" s="6"/>
-      <c r="H134" s="6" t="s">
+      <c r="D138" s="7"/>
+      <c r="E138" s="7"/>
+      <c r="F138" s="7"/>
+      <c r="H138" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="I134" s="6"/>
-      <c r="J134" s="6"/>
-      <c r="K134" s="6"/>
-      <c r="M134" s="6" t="s">
+      <c r="I138" s="7"/>
+      <c r="J138" s="7"/>
+      <c r="K138" s="7"/>
+      <c r="M138" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="N134" s="6"/>
-      <c r="O134" s="6"/>
-      <c r="P134" s="6"/>
-      <c r="R134" s="6" t="s">
+      <c r="N138" s="7"/>
+      <c r="O138" s="7"/>
+      <c r="P138" s="7"/>
+      <c r="R138" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="S134" s="6"/>
-      <c r="T134" s="6"/>
-      <c r="U134" s="6"/>
-    </row>
-    <row r="135" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C135" t="s">
-        <v>2</v>
-      </c>
-      <c r="D135" t="s">
-        <v>3</v>
-      </c>
-      <c r="E135" t="s">
-        <v>6</v>
-      </c>
-      <c r="F135" t="s">
-        <v>86</v>
-      </c>
-      <c r="H135" t="s">
-        <v>2</v>
-      </c>
-      <c r="I135" t="s">
-        <v>3</v>
-      </c>
-      <c r="J135" t="s">
-        <v>6</v>
-      </c>
-      <c r="K135" t="s">
-        <v>86</v>
-      </c>
-      <c r="M135" t="s">
-        <v>2</v>
-      </c>
-      <c r="N135" t="s">
-        <v>3</v>
-      </c>
-      <c r="O135" t="s">
-        <v>6</v>
-      </c>
-      <c r="P135" t="s">
-        <v>86</v>
-      </c>
-      <c r="R135" t="s">
-        <v>2</v>
-      </c>
-      <c r="S135" t="s">
-        <v>3</v>
-      </c>
-      <c r="T135" t="s">
-        <v>6</v>
-      </c>
-      <c r="U135" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="136" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C136" t="s">
-        <v>44</v>
-      </c>
-      <c r="D136" t="s">
-        <v>10</v>
-      </c>
-      <c r="E136" t="s">
-        <v>13</v>
-      </c>
-      <c r="H136" t="s">
-        <v>156</v>
-      </c>
-      <c r="I136" t="s">
-        <v>18</v>
-      </c>
-      <c r="J136" t="s">
-        <v>9</v>
-      </c>
-      <c r="M136" t="s">
-        <v>88</v>
-      </c>
-      <c r="N136" t="s">
-        <v>1</v>
-      </c>
-      <c r="O136" t="s">
-        <v>29</v>
-      </c>
-      <c r="R136" t="s">
-        <v>126</v>
-      </c>
-      <c r="S136" t="s">
-        <v>18</v>
-      </c>
-      <c r="T136" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="137" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C137" t="s">
-        <v>45</v>
-      </c>
-      <c r="D137" t="s">
-        <v>18</v>
-      </c>
-      <c r="E137" t="s">
-        <v>46</v>
-      </c>
-      <c r="H137" t="s">
-        <v>174</v>
-      </c>
-      <c r="I137" t="s">
-        <v>1</v>
-      </c>
-      <c r="J137" t="s">
-        <v>13</v>
-      </c>
-      <c r="M137" t="s">
-        <v>89</v>
-      </c>
-      <c r="N137" t="s">
-        <v>1</v>
-      </c>
-      <c r="O137" t="s">
-        <v>71</v>
-      </c>
-      <c r="R137" t="s">
-        <v>144</v>
-      </c>
-      <c r="S137" t="s">
-        <v>10</v>
-      </c>
-      <c r="T137" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="138" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C138" t="s">
-        <v>61</v>
-      </c>
-      <c r="D138" t="s">
-        <v>1</v>
-      </c>
-      <c r="E138" t="s">
-        <v>34</v>
-      </c>
-      <c r="H138" t="s">
-        <v>334</v>
-      </c>
-      <c r="I138" t="s">
-        <v>18</v>
-      </c>
-      <c r="J138" t="s">
-        <v>94</v>
-      </c>
-      <c r="M138" t="s">
-        <v>90</v>
-      </c>
-      <c r="N138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O138" t="s">
-        <v>13</v>
-      </c>
-      <c r="R138" t="s">
-        <v>154</v>
-      </c>
-      <c r="S138" t="s">
-        <v>1</v>
-      </c>
-      <c r="T138" t="s">
-        <v>9</v>
-      </c>
-      <c r="U138" t="s">
-        <v>115</v>
-      </c>
+      <c r="S138" s="7"/>
+      <c r="T138" s="7"/>
+      <c r="U138" s="7"/>
     </row>
     <row r="139" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C139" t="s">
-        <v>74</v>
+        <v>2</v>
       </c>
       <c r="D139" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E139" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="F139" t="s">
+        <v>86</v>
       </c>
       <c r="H139" t="s">
-        <v>335</v>
+        <v>2</v>
       </c>
       <c r="I139" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="J139" t="s">
-        <v>13</v>
+        <v>6</v>
+      </c>
+      <c r="K139" t="s">
+        <v>86</v>
       </c>
       <c r="M139" t="s">
-        <v>91</v>
+        <v>2</v>
       </c>
       <c r="N139" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="O139" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="P139" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="R139" t="s">
-        <v>158</v>
+        <v>2</v>
       </c>
       <c r="S139" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T139" t="s">
-        <v>150</v>
+        <v>6</v>
+      </c>
+      <c r="U139" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="140" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C140" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="D140" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E140" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H140" t="s">
-        <v>336</v>
+        <v>156</v>
       </c>
       <c r="I140" t="s">
+        <v>18</v>
+      </c>
+      <c r="J140" t="s">
+        <v>9</v>
+      </c>
+      <c r="M140" t="s">
+        <v>88</v>
+      </c>
+      <c r="N140" t="s">
         <v>1</v>
       </c>
-      <c r="J140" t="s">
-        <v>13</v>
-      </c>
-      <c r="M140" t="s">
-        <v>92</v>
-      </c>
-      <c r="N140" t="s">
-        <v>10</v>
-      </c>
       <c r="O140" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="R140" t="s">
-        <v>159</v>
+        <v>126</v>
       </c>
       <c r="S140" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="T140" t="s">
-        <v>160</v>
-      </c>
-      <c r="U140" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="141" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C141" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="D141" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E141" t="s">
+        <v>46</v>
+      </c>
+      <c r="H141" t="s">
+        <v>174</v>
+      </c>
+      <c r="I141" t="s">
+        <v>1</v>
+      </c>
+      <c r="J141" t="s">
         <v>13</v>
       </c>
       <c r="M141" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="N141" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O141" t="s">
-        <v>94</v>
-      </c>
-      <c r="P141" t="s">
-        <v>115</v>
+        <v>71</v>
       </c>
       <c r="R141" t="s">
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="S141" t="s">
         <v>10</v>
       </c>
       <c r="T141" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
     </row>
     <row r="142" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C142" t="s">
-        <v>312</v>
+        <v>61</v>
       </c>
       <c r="D142" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E142" t="s">
-        <v>48</v>
+        <v>34</v>
+      </c>
+      <c r="H142" t="s">
+        <v>334</v>
+      </c>
+      <c r="I142" t="s">
+        <v>18</v>
+      </c>
+      <c r="J142" t="s">
+        <v>94</v>
       </c>
       <c r="M142" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="N142" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O142" t="s">
         <v>13</v>
       </c>
       <c r="R142" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="S142" t="s">
         <v>1</v>
       </c>
       <c r="T142" t="s">
-        <v>13</v>
+        <v>9</v>
+      </c>
+      <c r="U142" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="143" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C143" t="s">
-        <v>313</v>
+        <v>74</v>
       </c>
       <c r="D143" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E143" t="s">
-        <v>23</v>
+        <v>7</v>
+      </c>
+      <c r="H143" t="s">
+        <v>335</v>
+      </c>
+      <c r="I143" t="s">
+        <v>18</v>
+      </c>
+      <c r="J143" t="s">
+        <v>13</v>
       </c>
       <c r="M143" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="N143" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="O143" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="P143" t="s">
         <v>115</v>
       </c>
       <c r="R143" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="S143" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="T143" t="s">
-        <v>13</v>
-      </c>
-      <c r="U143" t="s">
-        <v>115</v>
+        <v>150</v>
       </c>
     </row>
     <row r="144" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C144" t="s">
-        <v>375</v>
+        <v>77</v>
       </c>
       <c r="D144" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E144" t="s">
-        <v>376</v>
+        <v>7</v>
+      </c>
+      <c r="H144" t="s">
+        <v>336</v>
+      </c>
+      <c r="I144" t="s">
+        <v>1</v>
+      </c>
+      <c r="J144" t="s">
+        <v>13</v>
       </c>
       <c r="M144" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="N144" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="O144" t="s">
-        <v>23</v>
-      </c>
-      <c r="P144" t="s">
+        <v>9</v>
+      </c>
+      <c r="R144" t="s">
+        <v>159</v>
+      </c>
+      <c r="S144" t="s">
+        <v>4</v>
+      </c>
+      <c r="T144" t="s">
+        <v>160</v>
+      </c>
+      <c r="U144" t="s">
         <v>115</v>
-      </c>
-      <c r="R144" t="s">
-        <v>164</v>
-      </c>
-      <c r="S144" t="s">
-        <v>1</v>
-      </c>
-      <c r="T144" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="145" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C145" t="s">
-        <v>377</v>
+        <v>78</v>
       </c>
       <c r="D145" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E145" t="s">
-        <v>378</v>
+        <v>13</v>
       </c>
       <c r="M145" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="N145" t="s">
         <v>4</v>
       </c>
       <c r="O145" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="P145" t="s">
         <v>115</v>
       </c>
+      <c r="R145" t="s">
+        <v>161</v>
+      </c>
+      <c r="S145" t="s">
+        <v>10</v>
+      </c>
+      <c r="T145" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="146" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C146" t="s">
+        <v>312</v>
+      </c>
+      <c r="D146" t="s">
+        <v>18</v>
+      </c>
+      <c r="E146" t="s">
+        <v>48</v>
+      </c>
       <c r="M146" t="s">
+        <v>95</v>
+      </c>
+      <c r="N146" t="s">
+        <v>4</v>
+      </c>
+      <c r="O146" t="s">
+        <v>13</v>
+      </c>
+      <c r="R146" t="s">
+        <v>162</v>
+      </c>
+      <c r="S146" t="s">
+        <v>1</v>
+      </c>
+      <c r="T146" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="147" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C147" t="s">
+        <v>313</v>
+      </c>
+      <c r="D147" t="s">
+        <v>1</v>
+      </c>
+      <c r="E147" t="s">
+        <v>23</v>
+      </c>
+      <c r="M147" t="s">
+        <v>96</v>
+      </c>
+      <c r="N147" t="s">
+        <v>4</v>
+      </c>
+      <c r="O147" t="s">
+        <v>23</v>
+      </c>
+      <c r="P147" t="s">
+        <v>115</v>
+      </c>
+      <c r="R147" t="s">
+        <v>163</v>
+      </c>
+      <c r="S147" t="s">
+        <v>18</v>
+      </c>
+      <c r="T147" t="s">
+        <v>13</v>
+      </c>
+      <c r="U147" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="148" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C148" t="s">
+        <v>375</v>
+      </c>
+      <c r="D148" t="s">
+        <v>18</v>
+      </c>
+      <c r="E148" t="s">
+        <v>376</v>
+      </c>
+      <c r="M148" t="s">
+        <v>97</v>
+      </c>
+      <c r="N148" t="s">
+        <v>4</v>
+      </c>
+      <c r="O148" t="s">
+        <v>23</v>
+      </c>
+      <c r="P148" t="s">
+        <v>115</v>
+      </c>
+      <c r="R148" t="s">
+        <v>164</v>
+      </c>
+      <c r="S148" t="s">
+        <v>1</v>
+      </c>
+      <c r="T148" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="149" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C149" t="s">
+        <v>377</v>
+      </c>
+      <c r="D149" t="s">
+        <v>18</v>
+      </c>
+      <c r="E149" t="s">
+        <v>378</v>
+      </c>
+      <c r="M149" t="s">
+        <v>98</v>
+      </c>
+      <c r="N149" t="s">
+        <v>4</v>
+      </c>
+      <c r="O149" t="s">
+        <v>71</v>
+      </c>
+      <c r="P149" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="150" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="M150" t="s">
         <v>99</v>
       </c>
-      <c r="N146" t="s">
-        <v>4</v>
-      </c>
-      <c r="O146" t="s">
+      <c r="N150" t="s">
+        <v>4</v>
+      </c>
+      <c r="O150" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="147" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="M147" t="s">
+    <row r="151" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="M151" t="s">
         <v>101</v>
       </c>
-      <c r="N147" t="s">
-        <v>4</v>
-      </c>
-      <c r="O147" t="s">
+      <c r="N151" t="s">
+        <v>4</v>
+      </c>
+      <c r="O151" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="148" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="M148" t="s">
+    <row r="152" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="M152" t="s">
         <v>103</v>
       </c>
-      <c r="N148" t="s">
-        <v>4</v>
-      </c>
-      <c r="O148" t="s">
+      <c r="N152" t="s">
+        <v>4</v>
+      </c>
+      <c r="O152" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="149" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="M149" t="s">
+    <row r="153" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="M153" t="s">
         <v>104</v>
       </c>
-      <c r="N149" t="s">
-        <v>4</v>
-      </c>
-      <c r="O149" t="s">
+      <c r="N153" t="s">
+        <v>4</v>
+      </c>
+      <c r="O153" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="150" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C150" s="6" t="s">
+    <row r="154" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C154" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="D150" s="6"/>
-      <c r="E150" s="6"/>
-      <c r="F150" s="6"/>
-      <c r="H150" s="6" t="s">
+      <c r="D154" s="7"/>
+      <c r="E154" s="7"/>
+      <c r="F154" s="7"/>
+      <c r="H154" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="I150" s="6"/>
-      <c r="J150" s="6"/>
-      <c r="K150" s="6"/>
-      <c r="M150" t="s">
+      <c r="I154" s="7"/>
+      <c r="J154" s="7"/>
+      <c r="K154" s="7"/>
+      <c r="M154" t="s">
         <v>106</v>
       </c>
-      <c r="N150" t="s">
-        <v>18</v>
-      </c>
-      <c r="O150" t="s">
+      <c r="N154" t="s">
+        <v>18</v>
+      </c>
+      <c r="O154" t="s">
         <v>107</v>
       </c>
-      <c r="R150" s="6" t="s">
+      <c r="R154" s="7" t="s">
         <v>379</v>
       </c>
-      <c r="S150" s="6"/>
-      <c r="T150" s="6"/>
-      <c r="U150" s="6"/>
-    </row>
-    <row r="151" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C151" t="s">
-        <v>2</v>
-      </c>
-      <c r="D151" t="s">
-        <v>3</v>
-      </c>
-      <c r="E151" t="s">
-        <v>6</v>
-      </c>
-      <c r="F151" t="s">
-        <v>86</v>
-      </c>
-      <c r="H151" t="s">
-        <v>2</v>
-      </c>
-      <c r="I151" t="s">
-        <v>3</v>
-      </c>
-      <c r="J151" t="s">
-        <v>6</v>
-      </c>
-      <c r="K151" t="s">
-        <v>86</v>
-      </c>
-      <c r="M151" t="s">
-        <v>108</v>
-      </c>
-      <c r="N151" t="s">
-        <v>18</v>
-      </c>
-      <c r="O151" t="s">
-        <v>109</v>
-      </c>
-      <c r="R151" t="s">
-        <v>2</v>
-      </c>
-      <c r="S151" t="s">
-        <v>3</v>
-      </c>
-      <c r="T151" t="s">
-        <v>6</v>
-      </c>
-      <c r="U151" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="152" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C152" t="s">
-        <v>149</v>
-      </c>
-      <c r="D152" t="s">
-        <v>4</v>
-      </c>
-      <c r="E152" t="s">
-        <v>150</v>
-      </c>
-      <c r="H152" t="s">
-        <v>52</v>
-      </c>
-      <c r="I152" t="s">
-        <v>20</v>
-      </c>
-      <c r="J152" t="s">
-        <v>29</v>
-      </c>
-      <c r="M152" t="s">
-        <v>110</v>
-      </c>
-      <c r="N152" t="s">
-        <v>18</v>
-      </c>
-      <c r="O152" t="s">
-        <v>29</v>
-      </c>
-      <c r="R152" t="s">
-        <v>380</v>
-      </c>
-      <c r="S152" t="s">
-        <v>4</v>
-      </c>
-      <c r="T152" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="153" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C153" t="s">
-        <v>324</v>
-      </c>
-      <c r="D153" t="s">
-        <v>10</v>
-      </c>
-      <c r="E153" t="s">
-        <v>41</v>
-      </c>
-      <c r="H153" t="s">
-        <v>60</v>
-      </c>
-      <c r="I153" t="s">
-        <v>4</v>
-      </c>
-      <c r="J153" t="s">
-        <v>13</v>
-      </c>
-      <c r="M153" t="s">
-        <v>111</v>
-      </c>
-      <c r="N153" t="s">
-        <v>18</v>
-      </c>
-      <c r="O153" t="s">
-        <v>23</v>
-      </c>
-      <c r="R153" t="s">
-        <v>382</v>
-      </c>
-      <c r="S153" t="s">
-        <v>18</v>
-      </c>
-      <c r="T153" t="s">
-        <v>94</v>
-      </c>
-      <c r="U153" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="154" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C154" t="s">
-        <v>326</v>
-      </c>
-      <c r="D154" t="s">
-        <v>4</v>
-      </c>
-      <c r="E154" t="s">
-        <v>325</v>
-      </c>
-      <c r="H154" t="s">
-        <v>62</v>
-      </c>
-      <c r="I154" t="s">
-        <v>20</v>
-      </c>
-      <c r="J154" t="s">
-        <v>48</v>
-      </c>
-      <c r="M154" t="s">
-        <v>112</v>
-      </c>
-      <c r="N154" t="s">
-        <v>18</v>
-      </c>
-      <c r="O154" t="s">
-        <v>13</v>
-      </c>
-      <c r="R154" t="s">
-        <v>383</v>
-      </c>
-      <c r="S154" t="s">
-        <v>1</v>
-      </c>
-      <c r="T154" t="s">
-        <v>13</v>
-      </c>
+      <c r="S154" s="7"/>
+      <c r="T154" s="7"/>
+      <c r="U154" s="7"/>
     </row>
     <row r="155" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C155" t="s">
-        <v>327</v>
+        <v>2</v>
       </c>
       <c r="D155" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E155" t="s">
-        <v>332</v>
+        <v>6</v>
+      </c>
+      <c r="F155" t="s">
+        <v>86</v>
       </c>
       <c r="H155" t="s">
-        <v>82</v>
+        <v>2</v>
       </c>
       <c r="I155" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J155" t="s">
-        <v>29</v>
+        <v>6</v>
+      </c>
+      <c r="K155" t="s">
+        <v>86</v>
       </c>
       <c r="M155" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="N155" t="s">
         <v>18</v>
       </c>
       <c r="O155" t="s">
-        <v>29</v>
-      </c>
-      <c r="P155" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="R155" t="s">
-        <v>395</v>
+        <v>2</v>
       </c>
       <c r="S155" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="T155" t="s">
-        <v>48</v>
+        <v>6</v>
+      </c>
+      <c r="U155" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="156" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C156" t="s">
-        <v>328</v>
+        <v>149</v>
       </c>
       <c r="D156" t="s">
         <v>4</v>
       </c>
       <c r="E156" t="s">
-        <v>73</v>
+        <v>150</v>
       </c>
       <c r="H156" t="s">
-        <v>84</v>
+        <v>52</v>
       </c>
       <c r="I156" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="J156" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="M156" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="N156" t="s">
         <v>18</v>
       </c>
       <c r="O156" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="R156" t="s">
-        <v>396</v>
+        <v>380</v>
       </c>
       <c r="S156" t="s">
         <v>4</v>
       </c>
       <c r="T156" t="s">
-        <v>397</v>
+        <v>381</v>
       </c>
     </row>
     <row r="157" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C157" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="D157" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E157" t="s">
-        <v>333</v>
+        <v>41</v>
       </c>
       <c r="H157" t="s">
-        <v>167</v>
+        <v>60</v>
       </c>
       <c r="I157" t="s">
         <v>4</v>
       </c>
       <c r="J157" t="s">
-        <v>168</v>
+        <v>13</v>
       </c>
       <c r="M157" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="N157" t="s">
         <v>18</v>
       </c>
       <c r="O157" t="s">
-        <v>46</v>
-      </c>
-      <c r="R157" s="8" t="s">
-        <v>479</v>
-      </c>
-      <c r="S157" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="T157" s="8" t="s">
-        <v>467</v>
+        <v>23</v>
+      </c>
+      <c r="R157" t="s">
+        <v>382</v>
+      </c>
+      <c r="S157" t="s">
+        <v>18</v>
+      </c>
+      <c r="T157" t="s">
+        <v>94</v>
+      </c>
+      <c r="U157" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="158" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C158" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="D158" t="s">
         <v>4</v>
       </c>
       <c r="E158" t="s">
+        <v>325</v>
+      </c>
+      <c r="H158" t="s">
+        <v>62</v>
+      </c>
+      <c r="I158" t="s">
+        <v>20</v>
+      </c>
+      <c r="J158" t="s">
+        <v>48</v>
+      </c>
+      <c r="M158" t="s">
+        <v>112</v>
+      </c>
+      <c r="N158" t="s">
+        <v>18</v>
+      </c>
+      <c r="O158" t="s">
         <v>13</v>
       </c>
-      <c r="H158" t="s">
-        <v>169</v>
-      </c>
-      <c r="I158" t="s">
-        <v>18</v>
-      </c>
-      <c r="J158" t="s">
-        <v>7</v>
-      </c>
-      <c r="M158" t="s">
-        <v>117</v>
-      </c>
-      <c r="N158" t="s">
-        <v>18</v>
-      </c>
-      <c r="O158" t="s">
-        <v>34</v>
-      </c>
       <c r="R158" t="s">
-        <v>480</v>
+        <v>383</v>
       </c>
       <c r="S158" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="T158" t="s">
-        <v>481</v>
+        <v>13</v>
       </c>
     </row>
     <row r="159" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C159" t="s">
+        <v>327</v>
+      </c>
+      <c r="D159" t="s">
+        <v>20</v>
+      </c>
+      <c r="E159" t="s">
+        <v>332</v>
+      </c>
+      <c r="H159" t="s">
+        <v>82</v>
+      </c>
+      <c r="I159" t="s">
+        <v>10</v>
+      </c>
+      <c r="J159" t="s">
+        <v>29</v>
+      </c>
+      <c r="M159" t="s">
+        <v>113</v>
+      </c>
+      <c r="N159" t="s">
+        <v>18</v>
+      </c>
+      <c r="O159" t="s">
+        <v>29</v>
+      </c>
+      <c r="P159" t="s">
+        <v>115</v>
+      </c>
+      <c r="R159" t="s">
+        <v>395</v>
+      </c>
+      <c r="S159" t="s">
+        <v>18</v>
+      </c>
+      <c r="T159" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="160" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C160" t="s">
+        <v>328</v>
+      </c>
+      <c r="D160" t="s">
+        <v>4</v>
+      </c>
+      <c r="E160" t="s">
+        <v>73</v>
+      </c>
+      <c r="H160" t="s">
+        <v>84</v>
+      </c>
+      <c r="I160" t="s">
+        <v>4</v>
+      </c>
+      <c r="J160" t="s">
+        <v>13</v>
+      </c>
+      <c r="M160" t="s">
+        <v>114</v>
+      </c>
+      <c r="N160" t="s">
+        <v>18</v>
+      </c>
+      <c r="O160" t="s">
+        <v>71</v>
+      </c>
+      <c r="R160" t="s">
+        <v>396</v>
+      </c>
+      <c r="S160" t="s">
+        <v>4</v>
+      </c>
+      <c r="T160" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="161" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C161" t="s">
+        <v>329</v>
+      </c>
+      <c r="D161" t="s">
+        <v>1</v>
+      </c>
+      <c r="E161" t="s">
+        <v>333</v>
+      </c>
+      <c r="H161" t="s">
+        <v>167</v>
+      </c>
+      <c r="I161" t="s">
+        <v>4</v>
+      </c>
+      <c r="J161" t="s">
+        <v>168</v>
+      </c>
+      <c r="M161" t="s">
+        <v>116</v>
+      </c>
+      <c r="N161" t="s">
+        <v>18</v>
+      </c>
+      <c r="O161" t="s">
+        <v>46</v>
+      </c>
+      <c r="R161" s="9" t="s">
+        <v>479</v>
+      </c>
+      <c r="S161" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="T161" s="9" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="162" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C162" t="s">
+        <v>330</v>
+      </c>
+      <c r="D162" t="s">
+        <v>4</v>
+      </c>
+      <c r="E162" t="s">
+        <v>13</v>
+      </c>
+      <c r="H162" t="s">
+        <v>169</v>
+      </c>
+      <c r="I162" t="s">
+        <v>18</v>
+      </c>
+      <c r="J162" t="s">
+        <v>7</v>
+      </c>
+      <c r="M162" t="s">
+        <v>117</v>
+      </c>
+      <c r="N162" t="s">
+        <v>18</v>
+      </c>
+      <c r="O162" t="s">
+        <v>34</v>
+      </c>
+      <c r="R162" t="s">
+        <v>480</v>
+      </c>
+      <c r="S162" t="s">
+        <v>10</v>
+      </c>
+      <c r="T162" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="163" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C163" t="s">
         <v>331</v>
       </c>
-      <c r="D159" t="s">
-        <v>18</v>
-      </c>
-      <c r="E159" t="s">
+      <c r="D163" t="s">
+        <v>18</v>
+      </c>
+      <c r="E163" t="s">
         <v>13</v>
       </c>
-      <c r="H159" t="s">
+      <c r="H163" t="s">
         <v>354</v>
       </c>
-      <c r="I159" t="s">
+      <c r="I163" t="s">
         <v>1</v>
-      </c>
-      <c r="J159" t="s">
-        <v>69</v>
-      </c>
-      <c r="M159" t="s">
-        <v>118</v>
-      </c>
-      <c r="N159" t="s">
-        <v>18</v>
-      </c>
-      <c r="O159" t="s">
-        <v>13</v>
-      </c>
-      <c r="R159" t="s">
-        <v>482</v>
-      </c>
-      <c r="S159" t="s">
-        <v>4</v>
-      </c>
-      <c r="T159" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="160" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="H160" t="s">
-        <v>355</v>
-      </c>
-      <c r="I160" t="s">
-        <v>4</v>
-      </c>
-      <c r="J160" t="s">
-        <v>356</v>
-      </c>
-      <c r="M160" t="s">
-        <v>119</v>
-      </c>
-      <c r="N160" t="s">
-        <v>18</v>
-      </c>
-      <c r="O160" t="s">
-        <v>29</v>
-      </c>
-      <c r="R160" t="s">
-        <v>483</v>
-      </c>
-      <c r="S160" t="s">
-        <v>10</v>
-      </c>
-      <c r="T160" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="161" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H161" t="s">
-        <v>357</v>
-      </c>
-      <c r="I161" t="s">
-        <v>20</v>
-      </c>
-      <c r="J161" t="s">
-        <v>215</v>
-      </c>
-      <c r="M161" t="s">
-        <v>120</v>
-      </c>
-      <c r="N161" t="s">
-        <v>18</v>
-      </c>
-      <c r="O161" t="s">
-        <v>109</v>
-      </c>
-      <c r="R161" t="s">
-        <v>484</v>
-      </c>
-      <c r="S161" t="s">
-        <v>10</v>
-      </c>
-      <c r="T161" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="162" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H162" t="s">
-        <v>358</v>
-      </c>
-      <c r="I162" t="s">
-        <v>4</v>
-      </c>
-      <c r="J162" t="s">
-        <v>13</v>
-      </c>
-      <c r="M162" t="s">
-        <v>121</v>
-      </c>
-      <c r="N162" t="s">
-        <v>18</v>
-      </c>
-      <c r="O162" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="163" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H163" t="s">
-        <v>359</v>
-      </c>
-      <c r="I163" t="s">
-        <v>4</v>
       </c>
       <c r="J163" t="s">
         <v>69</v>
       </c>
       <c r="M163" t="s">
+        <v>118</v>
+      </c>
+      <c r="N163" t="s">
+        <v>18</v>
+      </c>
+      <c r="O163" t="s">
+        <v>13</v>
+      </c>
+      <c r="R163" t="s">
+        <v>482</v>
+      </c>
+      <c r="S163" t="s">
+        <v>4</v>
+      </c>
+      <c r="T163" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="164" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H164" t="s">
+        <v>355</v>
+      </c>
+      <c r="I164" t="s">
+        <v>4</v>
+      </c>
+      <c r="J164" t="s">
+        <v>356</v>
+      </c>
+      <c r="M164" t="s">
+        <v>119</v>
+      </c>
+      <c r="N164" t="s">
+        <v>18</v>
+      </c>
+      <c r="O164" t="s">
+        <v>29</v>
+      </c>
+      <c r="R164" t="s">
+        <v>483</v>
+      </c>
+      <c r="S164" t="s">
+        <v>10</v>
+      </c>
+      <c r="T164" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="165" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H165" t="s">
+        <v>357</v>
+      </c>
+      <c r="I165" t="s">
+        <v>20</v>
+      </c>
+      <c r="J165" t="s">
+        <v>215</v>
+      </c>
+      <c r="M165" t="s">
+        <v>120</v>
+      </c>
+      <c r="N165" t="s">
+        <v>18</v>
+      </c>
+      <c r="O165" t="s">
+        <v>109</v>
+      </c>
+      <c r="R165" t="s">
+        <v>484</v>
+      </c>
+      <c r="S165" t="s">
+        <v>10</v>
+      </c>
+      <c r="T165" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="166" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H166" t="s">
+        <v>358</v>
+      </c>
+      <c r="I166" t="s">
+        <v>4</v>
+      </c>
+      <c r="J166" t="s">
+        <v>13</v>
+      </c>
+      <c r="M166" t="s">
+        <v>121</v>
+      </c>
+      <c r="N166" t="s">
+        <v>18</v>
+      </c>
+      <c r="O166" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="167" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H167" t="s">
+        <v>359</v>
+      </c>
+      <c r="I167" t="s">
+        <v>4</v>
+      </c>
+      <c r="J167" t="s">
+        <v>69</v>
+      </c>
+      <c r="M167" t="s">
         <v>170</v>
       </c>
-      <c r="N163" t="s">
-        <v>4</v>
-      </c>
-      <c r="O163" t="s">
+      <c r="N167" t="s">
+        <v>4</v>
+      </c>
+      <c r="O167" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="164" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H164" t="s">
+    <row r="168" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H168" t="s">
         <v>360</v>
       </c>
-      <c r="I164" t="s">
-        <v>18</v>
-      </c>
-      <c r="J164" t="s">
+      <c r="I168" t="s">
+        <v>18</v>
+      </c>
+      <c r="J168" t="s">
         <v>48</v>
       </c>
-      <c r="M164" t="s">
+      <c r="M168" t="s">
         <v>172</v>
       </c>
-      <c r="N164" t="s">
+      <c r="N168" t="s">
         <v>20</v>
       </c>
-      <c r="O164" t="s">
+      <c r="O168" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="165" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H165" t="s">
+    <row r="169" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H169" t="s">
         <v>361</v>
       </c>
-      <c r="I165" t="s">
-        <v>18</v>
-      </c>
-      <c r="J165" t="s">
+      <c r="I169" t="s">
+        <v>18</v>
+      </c>
+      <c r="J169" t="s">
         <v>13</v>
       </c>
-      <c r="M165" t="s">
+      <c r="M169" t="s">
         <v>173</v>
       </c>
-      <c r="N165" t="s">
+      <c r="N169" t="s">
         <v>1</v>
       </c>
-      <c r="O165" t="s">
+      <c r="O169" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="166" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H166" t="s">
+    <row r="170" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H170" t="s">
         <v>362</v>
       </c>
-      <c r="I166" t="s">
-        <v>18</v>
-      </c>
-      <c r="J166" t="s">
+      <c r="I170" t="s">
+        <v>18</v>
+      </c>
+      <c r="J170" t="s">
         <v>48</v>
       </c>
-      <c r="M166" t="s">
+      <c r="M170" t="s">
         <v>191</v>
       </c>
-      <c r="N166" t="s">
-        <v>18</v>
-      </c>
-      <c r="O166" t="s">
+      <c r="N170" t="s">
+        <v>18</v>
+      </c>
+      <c r="O170" t="s">
         <v>102</v>
       </c>
-      <c r="R166" s="6" t="s">
+      <c r="R170" s="7" t="s">
         <v>384</v>
       </c>
-      <c r="S166" s="6"/>
-      <c r="T166" s="6"/>
-      <c r="U166" s="6"/>
-    </row>
-    <row r="167" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H167" t="s">
+      <c r="S170" s="7"/>
+      <c r="T170" s="7"/>
+      <c r="U170" s="7"/>
+    </row>
+    <row r="171" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H171" t="s">
         <v>363</v>
       </c>
-      <c r="I167" t="s">
-        <v>18</v>
-      </c>
-      <c r="J167" t="s">
+      <c r="I171" t="s">
+        <v>18</v>
+      </c>
+      <c r="J171" t="s">
         <v>13</v>
       </c>
-      <c r="M167" t="s">
+      <c r="M171" t="s">
         <v>337</v>
       </c>
-      <c r="N167" t="s">
-        <v>4</v>
-      </c>
-      <c r="O167" s="1" t="s">
+      <c r="N171" t="s">
+        <v>4</v>
+      </c>
+      <c r="O171" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="R167" t="s">
+      <c r="R171" t="s">
         <v>2</v>
       </c>
-      <c r="S167" t="s">
+      <c r="S171" t="s">
         <v>3</v>
       </c>
-      <c r="T167" t="s">
+      <c r="T171" t="s">
         <v>6</v>
       </c>
-      <c r="U167" t="s">
+      <c r="U171" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="168" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H168" t="s">
+    <row r="172" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H172" t="s">
         <v>364</v>
       </c>
-      <c r="I168" t="s">
+      <c r="I172" t="s">
         <v>10</v>
       </c>
-      <c r="J168" t="s">
+      <c r="J172" t="s">
         <v>365</v>
       </c>
-      <c r="K168" t="s">
+      <c r="K172" t="s">
         <v>115</v>
       </c>
-      <c r="M168" t="s">
+      <c r="M172" t="s">
         <v>338</v>
       </c>
-      <c r="N168" t="s">
-        <v>4</v>
-      </c>
-      <c r="O168" t="s">
+      <c r="N172" t="s">
+        <v>4</v>
+      </c>
+      <c r="O172" t="s">
         <v>339</v>
       </c>
-      <c r="R168" t="s">
+      <c r="R172" t="s">
         <v>385</v>
       </c>
-      <c r="S168" t="s">
+      <c r="S172" t="s">
         <v>1</v>
       </c>
-      <c r="T168" t="s">
+      <c r="T172" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="169" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H169" t="s">
+    <row r="173" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H173" t="s">
         <v>367</v>
-      </c>
-      <c r="I169" t="s">
-        <v>10</v>
-      </c>
-      <c r="J169" t="s">
-        <v>250</v>
-      </c>
-      <c r="K169" t="s">
-        <v>115</v>
-      </c>
-      <c r="M169" t="s">
-        <v>340</v>
-      </c>
-      <c r="N169" t="s">
-        <v>4</v>
-      </c>
-      <c r="O169" t="s">
-        <v>215</v>
-      </c>
-      <c r="R169" t="s">
-        <v>386</v>
-      </c>
-      <c r="S169" t="s">
-        <v>10</v>
-      </c>
-      <c r="T169" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="170" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H170" t="s">
-        <v>368</v>
-      </c>
-      <c r="I170" t="s">
-        <v>4</v>
-      </c>
-      <c r="J170" t="s">
-        <v>224</v>
-      </c>
-      <c r="M170" t="s">
-        <v>341</v>
-      </c>
-      <c r="N170" t="s">
-        <v>18</v>
-      </c>
-      <c r="O170" t="s">
-        <v>46</v>
-      </c>
-      <c r="R170" t="s">
-        <v>388</v>
-      </c>
-      <c r="S170" t="s">
-        <v>4</v>
-      </c>
-      <c r="T170" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="171" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H171" t="s">
-        <v>369</v>
-      </c>
-      <c r="I171" t="s">
-        <v>18</v>
-      </c>
-      <c r="J171" t="s">
-        <v>370</v>
-      </c>
-      <c r="M171" t="s">
-        <v>342</v>
-      </c>
-      <c r="N171" t="s">
-        <v>4</v>
-      </c>
-      <c r="O171" t="s">
-        <v>7</v>
-      </c>
-      <c r="R171" t="s">
-        <v>390</v>
-      </c>
-      <c r="S171" t="s">
-        <v>4</v>
-      </c>
-      <c r="T171" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="172" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H172" t="s">
-        <v>371</v>
-      </c>
-      <c r="I172" t="s">
-        <v>1</v>
-      </c>
-      <c r="J172" t="s">
-        <v>372</v>
-      </c>
-      <c r="M172" t="s">
-        <v>343</v>
-      </c>
-      <c r="N172" t="s">
-        <v>4</v>
-      </c>
-      <c r="O172" t="s">
-        <v>366</v>
-      </c>
-      <c r="R172" t="s">
-        <v>391</v>
-      </c>
-      <c r="S172" t="s">
-        <v>18</v>
-      </c>
-      <c r="T172" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="173" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="H173" t="s">
-        <v>373</v>
       </c>
       <c r="I173" t="s">
         <v>10</v>
       </c>
       <c r="J173" t="s">
-        <v>239</v>
+        <v>250</v>
+      </c>
+      <c r="K173" t="s">
+        <v>115</v>
       </c>
       <c r="M173" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="N173" t="s">
+        <v>4</v>
+      </c>
+      <c r="O173" t="s">
+        <v>215</v>
+      </c>
+      <c r="R173" t="s">
+        <v>386</v>
+      </c>
+      <c r="S173" t="s">
         <v>10</v>
       </c>
-      <c r="O173" t="s">
-        <v>9</v>
-      </c>
-      <c r="P173" t="s">
-        <v>115</v>
-      </c>
-      <c r="R173" t="s">
-        <v>392</v>
-      </c>
-      <c r="S173" t="s">
-        <v>18</v>
-      </c>
       <c r="T173" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="174" spans="8:21" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="174" spans="3:21" x14ac:dyDescent="0.25">
       <c r="H174" t="s">
-        <v>473</v>
+        <v>368</v>
       </c>
       <c r="I174" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="J174" t="s">
-        <v>13</v>
+        <v>224</v>
       </c>
       <c r="M174" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="N174" t="s">
         <v>18</v>
       </c>
       <c r="O174" t="s">
-        <v>236</v>
+        <v>46</v>
       </c>
       <c r="R174" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="S174" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="T174" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="175" spans="8:21" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="175" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H175" t="s">
+        <v>369</v>
+      </c>
+      <c r="I175" t="s">
+        <v>18</v>
+      </c>
+      <c r="J175" t="s">
+        <v>370</v>
+      </c>
       <c r="M175" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="N175" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="O175" t="s">
         <v>7</v>
       </c>
       <c r="R175" t="s">
+        <v>390</v>
+      </c>
+      <c r="S175" t="s">
+        <v>4</v>
+      </c>
+      <c r="T175" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="176" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="H176" t="s">
+        <v>371</v>
+      </c>
+      <c r="I176" t="s">
+        <v>1</v>
+      </c>
+      <c r="J176" t="s">
+        <v>372</v>
+      </c>
+      <c r="M176" t="s">
+        <v>343</v>
+      </c>
+      <c r="N176" t="s">
+        <v>4</v>
+      </c>
+      <c r="O176" t="s">
+        <v>366</v>
+      </c>
+      <c r="R176" t="s">
+        <v>391</v>
+      </c>
+      <c r="S176" t="s">
+        <v>18</v>
+      </c>
+      <c r="T176" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="177" spans="8:20" x14ac:dyDescent="0.25">
+      <c r="H177" t="s">
+        <v>373</v>
+      </c>
+      <c r="I177" t="s">
+        <v>10</v>
+      </c>
+      <c r="J177" t="s">
+        <v>239</v>
+      </c>
+      <c r="M177" t="s">
+        <v>344</v>
+      </c>
+      <c r="N177" t="s">
+        <v>10</v>
+      </c>
+      <c r="O177" t="s">
+        <v>9</v>
+      </c>
+      <c r="P177" t="s">
+        <v>115</v>
+      </c>
+      <c r="R177" t="s">
+        <v>392</v>
+      </c>
+      <c r="S177" t="s">
+        <v>18</v>
+      </c>
+      <c r="T177" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="178" spans="8:20" x14ac:dyDescent="0.25">
+      <c r="H178" t="s">
+        <v>473</v>
+      </c>
+      <c r="I178" t="s">
+        <v>18</v>
+      </c>
+      <c r="J178" t="s">
+        <v>13</v>
+      </c>
+      <c r="M178" t="s">
+        <v>345</v>
+      </c>
+      <c r="N178" t="s">
+        <v>18</v>
+      </c>
+      <c r="O178" t="s">
+        <v>236</v>
+      </c>
+      <c r="R178" t="s">
+        <v>393</v>
+      </c>
+      <c r="S178" t="s">
+        <v>18</v>
+      </c>
+      <c r="T178" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="179" spans="8:20" x14ac:dyDescent="0.25">
+      <c r="M179" t="s">
+        <v>346</v>
+      </c>
+      <c r="N179" t="s">
+        <v>18</v>
+      </c>
+      <c r="O179" t="s">
+        <v>7</v>
+      </c>
+      <c r="R179" t="s">
         <v>394</v>
       </c>
-      <c r="S175" t="s">
+      <c r="S179" t="s">
         <v>1</v>
       </c>
-      <c r="T175" t="s">
+      <c r="T179" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="176" spans="8:21" x14ac:dyDescent="0.25">
-      <c r="M176" t="s">
+    <row r="180" spans="8:20" x14ac:dyDescent="0.25">
+      <c r="M180" t="s">
         <v>347</v>
       </c>
-      <c r="N176" t="s">
+      <c r="N180" t="s">
         <v>20</v>
       </c>
-      <c r="O176" t="s">
+      <c r="O180" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="177" spans="13:15" x14ac:dyDescent="0.25">
-      <c r="M177" t="s">
+    <row r="181" spans="8:20" x14ac:dyDescent="0.25">
+      <c r="M181" t="s">
         <v>348</v>
       </c>
-      <c r="N177" t="s">
-        <v>18</v>
-      </c>
-      <c r="O177" t="s">
+      <c r="N181" t="s">
+        <v>18</v>
+      </c>
+      <c r="O181" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="178" spans="13:15" x14ac:dyDescent="0.25">
-      <c r="M178" t="s">
+    <row r="182" spans="8:20" x14ac:dyDescent="0.25">
+      <c r="M182" t="s">
         <v>349</v>
       </c>
-      <c r="N178" t="s">
-        <v>4</v>
-      </c>
-      <c r="O178" t="s">
+      <c r="N182" t="s">
+        <v>4</v>
+      </c>
+      <c r="O182" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="179" spans="13:15" x14ac:dyDescent="0.25">
-      <c r="M179" t="s">
+    <row r="183" spans="8:20" x14ac:dyDescent="0.25">
+      <c r="M183" t="s">
         <v>350</v>
       </c>
-      <c r="N179" t="s">
+      <c r="N183" t="s">
         <v>20</v>
       </c>
-      <c r="O179" t="s">
+      <c r="O183" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="180" spans="13:15" x14ac:dyDescent="0.25">
-      <c r="M180" t="s">
+    <row r="184" spans="8:20" x14ac:dyDescent="0.25">
+      <c r="M184" t="s">
         <v>352</v>
       </c>
-      <c r="N180" t="s">
-        <v>18</v>
-      </c>
-      <c r="O180" t="s">
+      <c r="N184" t="s">
+        <v>18</v>
+      </c>
+      <c r="O184" t="s">
         <v>353</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="R61:U61"/>
+    <mergeCell ref="R154:U154"/>
+    <mergeCell ref="R170:U170"/>
+    <mergeCell ref="C154:F154"/>
+    <mergeCell ref="H138:K138"/>
+    <mergeCell ref="C138:F138"/>
+    <mergeCell ref="H154:K154"/>
+    <mergeCell ref="R65:U65"/>
     <mergeCell ref="R4:U4"/>
-    <mergeCell ref="M134:P134"/>
+    <mergeCell ref="M138:P138"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="H4:K4"/>
     <mergeCell ref="M4:P4"/>
-    <mergeCell ref="C61:F61"/>
-    <mergeCell ref="H61:K61"/>
-    <mergeCell ref="M61:P61"/>
-    <mergeCell ref="R134:U134"/>
-    <mergeCell ref="R150:U150"/>
-    <mergeCell ref="R166:U166"/>
-    <mergeCell ref="C150:F150"/>
-    <mergeCell ref="H134:K134"/>
-    <mergeCell ref="C134:F134"/>
-    <mergeCell ref="H150:K150"/>
+    <mergeCell ref="C65:F65"/>
+    <mergeCell ref="H65:K65"/>
+    <mergeCell ref="M65:P65"/>
+    <mergeCell ref="R138:U138"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5988,29 +6082,29 @@
       <c r="B3" s="2"/>
     </row>
     <row r="5" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="I5" s="7" t="s">
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="I5" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
       <c r="M5" s="4"/>
-      <c r="N5" s="7" t="s">
+      <c r="N5" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="O5" s="7"/>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="7"/>
-      <c r="R5" s="7"/>
-      <c r="S5" s="7"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="8"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" t="s">

</xml_diff>

<commit_message>
fix: update inventario/db 2026-06-22 22:06:51
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\mbs_backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7A9A6A1-6F48-4AC5-A8B1-9F01594B08E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8641EAC-CE0C-4744-93BB-21576AD3751D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{20512AA4-7BE2-441B-A4C6-368DAF0E60CB}"/>
   </bookViews>
@@ -1652,7 +1652,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1671,12 +1671,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1690,7 +1684,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1701,7 +1695,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2392,30 +2385,30 @@
   </cols>
   <sheetData>
     <row r="4" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="H4" s="7" t="s">
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="H4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="M4" s="7" t="s">
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="M4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="R4" s="7" t="s">
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="R4" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="S4" s="7"/>
-      <c r="T4" s="7"/>
-      <c r="U4" s="7"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
     </row>
     <row r="5" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
@@ -3351,26 +3344,27 @@
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="R57" s="9" t="s">
+      <c r="R57" t="s">
         <v>486</v>
       </c>
-      <c r="S57" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="T57" s="9" t="s">
+      <c r="S57" t="s">
+        <v>18</v>
+      </c>
+      <c r="T57" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="R58" s="6" t="s">
+      <c r="R58" s="8" t="s">
         <v>490</v>
       </c>
-      <c r="S58" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="T58" s="6" t="s">
+      <c r="S58" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="T58" s="8" t="s">
         <v>23</v>
       </c>
+      <c r="U58" s="8"/>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="R59" t="s">
@@ -3390,30 +3384,30 @@
     </row>
     <row r="64" spans="1:21" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="65" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C65" s="7" t="s">
+      <c r="C65" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D65" s="7"/>
-      <c r="E65" s="7"/>
-      <c r="F65" s="7"/>
-      <c r="H65" s="7" t="s">
+      <c r="D65" s="6"/>
+      <c r="E65" s="6"/>
+      <c r="F65" s="6"/>
+      <c r="H65" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="I65" s="7"/>
-      <c r="J65" s="7"/>
-      <c r="K65" s="7"/>
-      <c r="M65" s="7" t="s">
+      <c r="I65" s="6"/>
+      <c r="J65" s="6"/>
+      <c r="K65" s="6"/>
+      <c r="M65" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="N65" s="7"/>
-      <c r="O65" s="7"/>
-      <c r="P65" s="7"/>
-      <c r="R65" s="7" t="s">
+      <c r="N65" s="6"/>
+      <c r="O65" s="6"/>
+      <c r="P65" s="6"/>
+      <c r="R65" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="S65" s="7"/>
-      <c r="T65" s="7"/>
-      <c r="U65" s="7"/>
+      <c r="S65" s="6"/>
+      <c r="T65" s="6"/>
+      <c r="U65" s="6"/>
     </row>
     <row r="66" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C66" t="s">
@@ -4029,13 +4023,13 @@
       <c r="J83" t="s">
         <v>13</v>
       </c>
-      <c r="R83" s="6" t="s">
+      <c r="R83" s="8" t="s">
         <v>493</v>
       </c>
-      <c r="S83" s="6" t="s">
+      <c r="S83" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="T83" s="6" t="s">
+      <c r="T83" s="8" t="s">
         <v>150</v>
       </c>
     </row>
@@ -4121,13 +4115,13 @@
       </c>
     </row>
     <row r="88" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C88" s="6" t="s">
+      <c r="C88" s="8" t="s">
         <v>491</v>
       </c>
-      <c r="D88" s="6" t="s">
+      <c r="D88" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="E88" s="6" t="s">
+      <c r="E88" s="8" t="s">
         <v>492</v>
       </c>
       <c r="H88" t="s">
@@ -4610,13 +4604,13 @@
       </c>
     </row>
     <row r="130" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="H130" s="9" t="s">
+      <c r="H130" t="s">
         <v>477</v>
       </c>
-      <c r="I130" s="9" t="s">
+      <c r="I130" t="s">
         <v>10</v>
       </c>
-      <c r="J130" s="9" t="s">
+      <c r="J130" t="s">
         <v>13</v>
       </c>
     </row>
@@ -4654,42 +4648,42 @@
       </c>
     </row>
     <row r="134" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="H134" s="6" t="s">
+      <c r="H134" s="8" t="s">
         <v>494</v>
       </c>
-      <c r="I134" s="6" t="s">
+      <c r="I134" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="J134" s="6" t="s">
+      <c r="J134" s="8" t="s">
         <v>332</v>
       </c>
-      <c r="K134" s="6"/>
+      <c r="K134" s="8"/>
     </row>
     <row r="138" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C138" s="7" t="s">
+      <c r="C138" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D138" s="7"/>
-      <c r="E138" s="7"/>
-      <c r="F138" s="7"/>
-      <c r="H138" s="7" t="s">
+      <c r="D138" s="6"/>
+      <c r="E138" s="6"/>
+      <c r="F138" s="6"/>
+      <c r="H138" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="I138" s="7"/>
-      <c r="J138" s="7"/>
-      <c r="K138" s="7"/>
-      <c r="M138" s="7" t="s">
+      <c r="I138" s="6"/>
+      <c r="J138" s="6"/>
+      <c r="K138" s="6"/>
+      <c r="M138" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="N138" s="7"/>
-      <c r="O138" s="7"/>
-      <c r="P138" s="7"/>
-      <c r="R138" s="7" t="s">
+      <c r="N138" s="6"/>
+      <c r="O138" s="6"/>
+      <c r="P138" s="6"/>
+      <c r="R138" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="S138" s="7"/>
-      <c r="T138" s="7"/>
-      <c r="U138" s="7"/>
+      <c r="S138" s="6"/>
+      <c r="T138" s="6"/>
+      <c r="U138" s="6"/>
     </row>
     <row r="139" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C139" t="s">
@@ -5136,18 +5130,18 @@
       </c>
     </row>
     <row r="154" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C154" s="7" t="s">
+      <c r="C154" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="D154" s="7"/>
-      <c r="E154" s="7"/>
-      <c r="F154" s="7"/>
-      <c r="H154" s="7" t="s">
+      <c r="D154" s="6"/>
+      <c r="E154" s="6"/>
+      <c r="F154" s="6"/>
+      <c r="H154" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I154" s="7"/>
-      <c r="J154" s="7"/>
-      <c r="K154" s="7"/>
+      <c r="I154" s="6"/>
+      <c r="J154" s="6"/>
+      <c r="K154" s="6"/>
       <c r="M154" t="s">
         <v>106</v>
       </c>
@@ -5157,12 +5151,12 @@
       <c r="O154" t="s">
         <v>107</v>
       </c>
-      <c r="R154" s="7" t="s">
+      <c r="R154" s="6" t="s">
         <v>379</v>
       </c>
-      <c r="S154" s="7"/>
-      <c r="T154" s="7"/>
-      <c r="U154" s="7"/>
+      <c r="S154" s="6"/>
+      <c r="T154" s="6"/>
+      <c r="U154" s="6"/>
     </row>
     <row r="155" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C155" t="s">
@@ -5435,13 +5429,13 @@
       <c r="O161" t="s">
         <v>46</v>
       </c>
-      <c r="R161" s="9" t="s">
+      <c r="R161" t="s">
         <v>479</v>
       </c>
-      <c r="S161" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="T161" s="9" t="s">
+      <c r="S161" t="s">
+        <v>4</v>
+      </c>
+      <c r="T161" t="s">
         <v>467</v>
       </c>
     </row>
@@ -5678,12 +5672,12 @@
       <c r="O170" t="s">
         <v>102</v>
       </c>
-      <c r="R170" s="7" t="s">
+      <c r="R170" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="S170" s="7"/>
-      <c r="T170" s="7"/>
-      <c r="U170" s="7"/>
+      <c r="S170" s="6"/>
+      <c r="T170" s="6"/>
+      <c r="U170" s="6"/>
     </row>
     <row r="171" spans="3:21" x14ac:dyDescent="0.25">
       <c r="H171" t="s">
@@ -6006,12 +6000,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="R154:U154"/>
-    <mergeCell ref="R170:U170"/>
-    <mergeCell ref="C154:F154"/>
-    <mergeCell ref="H138:K138"/>
-    <mergeCell ref="C138:F138"/>
-    <mergeCell ref="H154:K154"/>
     <mergeCell ref="R65:U65"/>
     <mergeCell ref="R4:U4"/>
     <mergeCell ref="M138:P138"/>
@@ -6022,6 +6010,12 @@
     <mergeCell ref="H65:K65"/>
     <mergeCell ref="M65:P65"/>
     <mergeCell ref="R138:U138"/>
+    <mergeCell ref="R154:U154"/>
+    <mergeCell ref="R170:U170"/>
+    <mergeCell ref="C154:F154"/>
+    <mergeCell ref="H138:K138"/>
+    <mergeCell ref="C138:F138"/>
+    <mergeCell ref="H154:K154"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6082,29 +6076,29 @@
       <c r="B3" s="2"/>
     </row>
     <row r="5" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="I5" s="8" t="s">
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="I5" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
       <c r="M5" s="4"/>
-      <c r="N5" s="8" t="s">
+      <c r="N5" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="8"/>
-      <c r="S5" s="8"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="7"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" t="s">

</xml_diff>